<commit_message>
docs(ejecucion): unifica los reportes de todos los módulos en 04, 05 y 06
Exportar CSV, Importar Excel y Suscripciones pasan a los reportes globales
de ejecución, defectos y resumen (md y xlsx), junto con Deudas y Navegación:
una sola tabla de 567 casos, un solo índice de defectos (DEF-029 a DEF-036,
con el mismo formato), métricas, quién ejecutó cada caso (IA o equipo),
criterios de salida y desvíos. Los casos que no son PASSED de Deudas y
Navegación ahora muestran también lo esperado.

Borra los reportes sueltos por módulo (-exp, -imp, -sus) y actualiza el README.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega-2/05-reportes-de-defectos.xlsx
+++ b/entrega-2/05-reportes-de-defectos.xlsx
@@ -9,6 +9,13 @@
   <sheets>
     <sheet name="Index" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="DEF-029" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="DEF-030" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="DEF-031" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="DEF-032" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="DEF-033" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="DEF-034" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="DEF-035" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="DEF-036" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -67,7 +74,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -81,11 +88,25 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -101,6 +122,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -468,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -483,7 +519,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Biyu · Entrega 2 · Defect reports</t>
+          <t>Biyu · Entrega 2 · Defect reports · Deudas, Navegación, Exportar CSV, Importar Excel y Suscripciones</t>
         </is>
       </c>
     </row>
@@ -558,6 +594,265 @@
       <c r="G3" s="3" t="inlineStr">
         <is>
           <t>— (sin issue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>DEF-030</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Tocar fuera de la hoja «Exportar movimientos» no la cierra</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Abierto · se reproduce el 2026-10-27</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>CP-EXP-062 (también quita valor a CP-EXP-070)</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>US-47 · Exportar movimientos a CSV (CA-23)</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>sin issue</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>DEF-031</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>«Atrás» y «Adelante» del navegador cambian la URL pero la hoja de exportar queda abierta</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Abierto · se reproduce el 2026-10-27</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>CP-EXP-063 y CP-EXP-065</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>US-47 · Exportar movimientos a CSV (CA-24 y requisito «todo cambio de URL»)</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>sin issue</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>DEF-032</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>«Atrás» durante «Exportando…» no cancela la exportación: el archivo se descarga igual</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Abierto · se reproduce el 2026-10-27</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>CP-EXP-064</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>US-47 · Exportar movimientos a CSV (CA-24)</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>sin issue</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>DEF-033</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>La tarjeta de una fila lista muestra la categoría y la cuenta como están escritas en el archivo, no como se llaman en Biyu</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Abierto · se reproduce el 2026-10-27</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>CP-IMP-052</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>US-76 · Revisión de filas (CA-5)</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>sin issue</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>DEF-034</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Operar sobre la suscripción de otro usuario responde HTTP 500 en lugar de 404</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Abierto · se reproduce el 2026-10-27</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>CP-SUS-094, CP-SUS-100, CP-SUS-107 y CP-SUS-129</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>US-56 · CA-9, US-57 · CA-7, US-58 · CA-9 y US-59 (Pausar, reanudar, cancelar y editar: par de autorización)</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>sin issue</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>DEF-035</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Sin sesión, la API responde HTTP 401 y los casos esperan 403</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Abierto · se reproduce el 2026-10-27</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>CP-SUS-065, CP-SUS-066, CP-SUS-095, CP-SUS-101, CP-SUS-108 y CP-SUS-130</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>US-52 · CA-13 y US-56 · CA-9, US-57 · CA-7, US-58 · CA-9, US-59 (rol anon)</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>sin issue</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>DEF-036</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>La vista previa del calendario no marca con data-blocked="false" las filas que no están bloqueadas</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Abierto · se reproduce el 2026-10-27</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>CP-SUS-157</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>US-61 · Vista previa del calendario al dar de alta una suscripción</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>sin issue</t>
         </is>
       </c>
     </row>
@@ -565,6 +860,15 @@
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId7"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -755,4 +1059,1278 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31.83" customWidth="1" min="1" max="1"/>
+    <col width="63.66" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>[DEF-030] Tocar fuera de la hoja «Exportar movimientos» no la cierra</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Description / Overview</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Tocar fuera de la hoja «Exportar movimientos» no la cierra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5" ht="45" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Reproduction Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>1- Abrir la app e iniciar sesión con un usuario de prueba. Si aparece la configuración inicial, tocar «Saltear» en sus 4 pasos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>2- Crear un gasto con fecha en septiembre de 2026 y abrir en el navegador /transactions?period=2026-09.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>3- Tocar «Exportar» arriba a la derecha: se abre la hoja «Exportar movimientos».</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>4- Hacer clic sobre el fondo oscuro, fuera de la hoja (por ejemplo, en la esquina superior izquierda de la pantalla).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>5- Mirar si la hoja sigue abierta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Expected Behavior</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>CA-23 / CP-EXP-062: tocar fuera de la hoja la cierra sin descargar nada y la URL conserva ?period=2026-09 (mientras no esté en «Exportando…»).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Actual Behavior</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>La hoja sigue abierta. El elemento que recibe el clic en esa posición es el div de fondo (clases fixed inset-0 -z-10, aria-hidden="true"), no el contenedor de la hoja. Solo «Cancelar» y Escape la cierran.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Incidence / Severity / Probability of reproduction</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Severidad Media - no se pierden datos y la hoja se puede cerrar con «Cancelar» o Escape, pero se incumple CA-23 y un gesto habitual no hace nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>100 % (3 de 3 ejecuciones).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Story and Acceptance Criteria affected</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>US-47 · CA-23: «Tocar fuera de la hoja la cierra sin descargar» (CP-EXP-062). Además, CP-EXP-070 («tocar fuera no cierra la hoja durante Exportando») pasa sin probar nada mientras este defecto siga abierto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Browsers tested</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Chromium (Playwright 1.63), ventana de 420 × 900. No se probó en otros navegadores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63), reloj fijado en 09/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
+    <row r="24" ht="240" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>- Defect ID: DEF-030
+- Estado: Abierto · se reproduce el 2026-10-27
+- Issue de GitHub: sin issue
+- Caso de prueba: CP-EXP-062 (también quita valor a CP-EXP-070)
+- Encontrado en: ejecución de CP-EXP-062 (Entrega 2).
+- Reportó: Claude Code (IA), supervisado por Santiago
+- Evidencia: Observado en la corrida de CP-EXP-062: la hoja sigue abierta tras el clic; document.elementFromPoint(5, 5) = DIV.fixed.inset-0.-z-10.bg-[rgba(43,30,25,0.32)], aria-hidden=true
+- Causa probable: en src/components/transactions/ExportTransactionsDialog.tsx el cierre por clic exige e.target === e.currentTarget, pero el div de fondo es hijo del contenedor y cubre toda la pantalla: recibe el clic y el destino nunca coincide. No se corrigió nada.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31.83" customWidth="1" min="1" max="1"/>
+    <col width="63.66" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>[DEF-031] «Atrás» y «Adelante» del navegador cambian la URL pero la hoja de exportar queda abierta</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="45" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Description / Overview</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Con la hoja «Exportar movimientos» abierta, «Atrás» y «Adelante» del navegador cambian el período de la URL pero la hoja no se cierra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Reproduction Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>1- Abrir la app e iniciar sesión con un usuario de prueba (con la configuración inicial salteada).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1">
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>2- Abrir en el navegador /transactions?period=2026-08.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>3- Tocar el botón de mes siguiente: la URL pasa a ?period=2026-09.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>4- Tocar «Exportar»: se abre la hoja.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>5- Hacer clic en «Atrás» del navegador y mirar la URL y la hoja. (Para CP-EXP-065: abrir la hoja en agosto, después de haber vuelto desde septiembre, y hacer clic en «Adelante».)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Expected Behavior</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>CA-24 / CP-EXP-063 y 065: la hoja se cierra, la URL pasa a ?period=2026-08 (con «Adelante», a ?period=2026-09) y no se descarga archivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Actual Behavior</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>La URL cambia al período anterior (o al siguiente) y la hoja sigue abierta. El evento popstate sí se dispara (verificado en 3 de 3 repeticiones), pero la hoja no se cierra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Incidence / Severity / Probability of reproduction</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Severidad Media - no se pierden ni se duplican datos, pero la hoja queda sobre otro período y el usuario puede descargar un mes distinto del que ve en la URL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>100 % (3 de 3 ejecuciones).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18" ht="45" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Story and Acceptance Criteria affected</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>US-47 · CA-24: «Si cambia la URL o se presiona Atrás, la hoja se cierra y no se descarga nada», y el requisito «todo cambio de URL cierra la hoja» (CP-EXP-063 y CP-EXP-065).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Browsers tested</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Chromium (Playwright 1.63). No se probó en otros navegadores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63), reloj fijado en 09/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
+    <row r="24" ht="240" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>- Defect ID: DEF-031
+- Estado: Abierto · se reproduce el 2026-10-27
+- Issue de GitHub: sin issue
+- Caso de prueba: CP-EXP-063 y CP-EXP-065
+- Encontrado en: ejecución de CP-EXP-063 y CP-EXP-065 (Entrega 2).
+- Reportó: Claude Code (IA), supervisado por Santiago
+- Evidencia: Observado en las corridas de CP-EXP-063 y CP-EXP-065: URL cambiada con la hoja abierta; log de popstate: ['popstate@?period=2026-08']
+- Causa no determinada. En ExportTransactionsDialog.tsx hay un efecto que cierra la hoja cuando cambia location.key y un oyente de popstate; ninguno logra cerrarla. Hipótesis sin confirmar: el efecto que reinicia initialLocationKeyRef cuando cambia location.key corre antes del que compara la clave y la deja siempre igual. No se corrigió nada.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31.83" customWidth="1" min="1" max="1"/>
+    <col width="63.66" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>[DEF-032] «Atrás» durante «Exportando…» no cancela la exportación: el archivo se descarga igual</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Description / Overview</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>«Atrás» durante «Exportando…» no cancela la exportación: el archivo se descarga igual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Reproduction Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>1- Abrir la app e iniciar sesión con un usuario de prueba que tenga un gasto de septiembre de 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>2- Abrir /transactions?period=2026-08, tocar el mes siguiente (URL ?period=2026-09) y tocar «Exportar».</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>3- Demorar unos segundos las respuestas de /rest/v1/transactions (en las pruebas, 3 s con Playwright; en DevTools, «1 kbit/s» y latencia 2000 ms).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>4- Tocar «Descargar CSV»: el botón pasa a «Exportando…».</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>5- Hacer clic en «Atrás» del navegador y esperar a que termine la demora.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Expected Behavior</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>CA-24 / CP-EXP-064 (paso 22): la exportación se cancela; no aparece ningún archivo ni aviso de éxito.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Actual Behavior</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Al terminar la lectura se descarga biyu-movimientos-2026-09.csv y aparece el aviso «Exportamos 1 movimiento» (1 descarga y 1 aviso), con el usuario ya en ?period=2026-08.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Incidence / Severity / Probability of reproduction</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Severidad Media - se descarga un archivo que el usuario ya había abandonado; no afecta datos guardados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>100 % (2 de 2 ejecuciones).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Story and Acceptance Criteria affected</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>US-47 · CA-24: «Atrás durante Exportando… cancela la descarga» (CP-EXP-064).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Browsers tested</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Chromium (Playwright 1.63). No se probó en otros navegadores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63), reloj fijado en 09/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
+    <row r="24" ht="180" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>- Defect ID: DEF-032
+- Estado: Abierto · se reproduce el 2026-10-27
+- Issue de GitHub: sin issue
+- Caso de prueba: CP-EXP-064
+- Encontrado en: ejecución de CP-EXP-064 (Entrega 2).
+- Reportó: Claude Code (IA), supervisado por Santiago
+- Evidencia: Observado en la corrida de CP-EXP-064: aviso de éxito en el período anterior; descargas registradas por el navegador = 1
+- Relacionado con DEF-031: el cierre por «Atrás» no llega a abortar la exportación en curso (AbortController). No se investigó a fondo. No se corrigió nada.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31.83" customWidth="1" min="1" max="1"/>
+    <col width="63.66" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="45" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>[DEF-033] La tarjeta de una fila lista muestra la categoría y la cuenta como están escritas en el archivo, no como se llaman en Biyu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="75" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Description / Overview</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>En la Revisión del importador, la tarjeta de una fila «Lista» muestra el texto de la categoría y de la cuenta tal cual está en el Excel (por ejemplo «educación» y «efectivo»), en lugar del nombre con el que existen en Biyu («Educación» y «Efectivo»).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5" ht="45" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Reproduction Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>1- Abrir la app e iniciar sesión con un usuario de prueba (con la configuración inicial salteada) y tocar «Importar desde Excel».</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>2- Armar un .xlsx con los encabezados de la plantilla y una fila: fecha 01/09/2026, Tipo « gasto » (con espacios), Monto 10, Moneda «usd», Tipo de cambio 1450, Categoría «  educación  », Cuenta «  efectivo  », Cuotas 1, Nota «Coincidencia».</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>3- Tocar «Elegir archivo .xlsx» y elegir el archivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>4- Mirar la tarjeta «Fila 2» de la Revisión.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Expected Behavior</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>CP-IMP-052 (paso 10): «Fila 2» está «Lista» y muestra «Gasto», «US$10,00», «Educación», «Efectivo» y «TC 1.450,00».</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Actual Behavior</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>La fila está «Lista» (la coincidencia sin distinguir mayúsculas ni espacios funciona) pero la tarjeta dice «01/09/2026 · Gasto · educación · efectivo · TC 1.450,00 US$10,00»: muestra el texto del archivo, no los nombres de Biyu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Incidence / Severity / Probability of reproduction</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Severidad Baja - las filas se importan bien (se asocian a la categoría y cuenta correctas); solo cambia lo que se muestra antes de confirmar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1">
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>100 % (1 de 1 ejecución).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Story and Acceptance Criteria affected</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>US-76 · CA-5: coincidencia de nombres sin distinguir mayúsculas ni espacios, con la tarjeta mostrando los nombres de Biyu (CP-IMP-052).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Browsers tested</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Chromium (Playwright 1.63). No se probó en otros navegadores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23" ht="165" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>- Defect ID: DEF-033
+- Estado: Abierto · se reproduce el 2026-10-27
+- Issue de GitHub: sin issue
+- Caso de prueba: CP-IMP-052
+- Encontrado en: ejecución de CP-IMP-052 (Entrega 2).
+- Reportó: Claude Code (IA), supervisado por Santiago
+- Evidencia: Texto de la tarjeta import-row-2 en la corrida de CP-IMP-052
+- Causa probable: la tarjeta arma el detalle con el texto leído del archivo y no con el nombre del catálogo que resolvió la fila. No se investigó a fondo ni se corrigió nada.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31.83" customWidth="1" min="1" max="1"/>
+    <col width="63.66" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>[DEF-034] Operar sobre la suscripción de otro usuario responde HTTP 500 en lugar de 404</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="75" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Description / Overview</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Cuando un usuario llama a pause_subscription, resume_subscription, cancel_subscription o update_subscription con el identificador de una suscripción de otro usuario, la API rechaza la operación (P0002 «Suscripción no encontrada») pero con HTTP 500 en lugar de 404.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Reproduction Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>1- Crear dos usuarios de prueba, A y B, con la configuración inicial salteada, y obtener el token de cada uno (PR-04).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>2- Con el token de B, crear una suscripción (POST /rest/v1/rpc/create_subscription) y guardar su id.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>3- Con el token de A, enviar POST /rest/v1/rpc/pause_subscription con body {"p_subscription_id":"&lt;id de B&gt;"}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>4- Mirar el código HTTP y el cuerpo. Repetir con resume_subscription (sobre una pausada), cancel_subscription y update_subscription.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Expected Behavior</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Los casos esperan HTTP 404 con "code": "P0002" y "message": "Suscripción no encontrada".</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Actual Behavior</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>HTTP 500 con {"code":"P0002","details":null,"hint":null,"message":"Suscripción no encontrada"}. El código y el mensaje coinciden; cambia el HTTP. La suscripción de B no se modifica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Incidence / Severity / Probability of reproduction</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Severidad Baja - la operación se rechaza bien y no se filtra ningún dato, pero un «no encontrado» se informa como error del servidor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1">
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>100 % (4 de 4 ejecuciones).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Story and Acceptance Criteria affected</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>US-56 · CA-9, US-57 · CA-7, US-58 · CA-9: «otro usuario recibe P0002 "Suscripción no encontrada"»; los casos agregan el HTTP 404.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Browsers tested</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>No aplica: llamada directa a la API.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21" ht="45" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63) · Edge Functions locales levantadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23" ht="225" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>- Defect ID: DEF-034
+- Estado: Abierto · se reproduce el 2026-10-27
+- Issue de GitHub: sin issue
+- Caso de prueba: CP-SUS-094, CP-SUS-100, CP-SUS-107 y CP-SUS-129
+- Encontrado en: ejecución de CP-SUS-094, 100, 107 y 129 (Entrega 2).
+- Reportó: Claude Code (IA), supervisado por Santiago
+- Evidencia: Respuesta de la API en las corridas de CP-SUS-094, 100, 107 y 129
+- Causa probable: PostgREST solo traduce a 4xx algunos códigos de error y P0002 no está entre ellos; hace falta un código propio (por ejemplo PT404) en la función. No se investigó a fondo ni se corrigió nada. Decisión pendiente: cambiar la función o el resultado esperado de los casos.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31.83" customWidth="1" min="1" max="1"/>
+    <col width="63.66" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>[DEF-035] Sin sesión, la API responde HTTP 401 y los casos esperan 403</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="60" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Description / Overview</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Las llamadas a las funciones y la lectura de la tabla de suscripciones con la clave anónima (sin sesión) se rechazan con "code": "42501" como pide el caso, pero con HTTP 401 y no con 403.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5" ht="45" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Reproduction Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>1- Con la clave anónima como apikey y como Bearer, enviar POST /rest/v1/rpc/create_subscription con un body válido (o GET /rest/v1/subscriptions?select=*).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>2- Mirar el código HTTP y el cuerpo. Repetir con pause_subscription, resume_subscription, cancel_subscription y update_subscription.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Expected Behavior</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden con "code": "42501" («permission denied for function …» o «… for table subscriptions»).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Actual Behavior</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>HTTP 401 con "code": "42501" y el mismo mensaje de permiso denegado. No se crea ni se lee nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Incidence / Severity / Probability of reproduction</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Severidad Baja - el acceso se deniega correctamente; solo cambia el número HTTP respecto del caso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1">
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>100 % (6 de 6 ejecuciones).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Story and Acceptance Criteria affected</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>US-52 · CA-13 y los pares de autorización de US-56 a US-59: «sin sesión (anon) recibe 42501».</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Browsers tested</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>No aplica: llamada directa a la API.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63) · Edge Functions locales levantadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21" ht="210" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>- Defect ID: DEF-035
+- Estado: Abierto · se reproduce el 2026-10-27
+- Issue de GitHub: sin issue
+- Caso de prueba: CP-SUS-065, CP-SUS-066, CP-SUS-095, CP-SUS-101, CP-SUS-108 y CP-SUS-130
+- Encontrado en: ejecución de CP-SUS-065, 066, 095, 101, 108 y 130 (Entrega 2).
+- Reportó: Claude Code (IA), supervisado por Santiago
+- Evidencia: Respuesta de la API en las corridas de los seis casos
+- Parece un error de los casos: PostgREST responde 401 al rol anónimo (el mismo comportamiento se vio en CP-DEU-029 y CP-DEU-108). No se corrigió nada. Decisión pendiente: corregir el HTTP esperado en los seis casos.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31.83" customWidth="1" min="1" max="1"/>
+    <col width="63.66" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>[DEF-036] La vista previa del calendario no marca con data-blocked="false" las filas que no están bloqueadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="60" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Description / Overview</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>En «Se cargan al guardar», la fila de un mes sin bloqueo no tiene el atributo data-blocked; el caso espera data-blocked="false". La fila bloqueada sí lleva data-blocked="true" y el texto «Sin tipo de cambio: se carga cuando lo cargues».</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5" ht="45" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Reproduction Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>1- Abrir la app e iniciar sesión con un usuario de prueba y cargar solo el tipo de cambio del mes de hace 2 meses (1200,00) en Ajustes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>2- Abrir /subscriptions/new, elegir USD, escribir monto 20 y día de cobro 28, y poner como mes de inicio el de hace 2 meses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>3- Con las herramientas de desarrollo, mirar los atributos de las filas subscription-form-preview-due-item de cada mes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Expected Behavior</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>La fila del mes con tipo de cambio tiene data-blocked="false" y la del mes sin tipo de cambio data-blocked="true" (CP-SUS-157, paso 11).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Actual Behavior</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>La fila del mes con tipo de cambio no tiene el atributo data-blocked; la del mes sin tipo de cambio sí lo tiene en "true" y muestra el texto esperado. El resumen dice «Al guardar se carga 1 gasto de USD 20,00.»</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Incidence / Severity / Probability of reproduction</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Severidad Baja - no afecta a quien usa la app; solo la automatización que busca el atributo "false".</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1">
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>100 % (1 de 1 ejecución).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Story and Acceptance Criteria affected</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>US-61 · CA-5 (vista previa con meses bloqueados por falta de tipo de cambio).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Browsers tested</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Chromium (Playwright 1.63). No se probó en otros navegadores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63) · Edge Functions locales levantadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22" ht="165" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>- Defect ID: DEF-036
+- Estado: Abierto · se reproduce el 2026-10-27
+- Issue de GitHub: sin issue
+- Caso de prueba: CP-SUS-157
+- Encontrado en: ejecución de CP-SUS-157 (Entrega 2).
+- Reportó: Claude Code (IA), supervisado por Santiago
+- Evidencia: Observaciones de la corrida de CP-SUS-157
+- En src/components/subscriptions/SubscriptionPreview.tsx el atributo se escribe como data-blocked={row.blockedBy ? 'true' : undefined}. Parece un error del caso, o un atributo de automatización por completar. No se corrigió nada.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(ejecucion): suma 44 casos de Deudas (039 a 093) y DEF-037 a los reportes unificados
Ejecución con IA (Claude Code, supervisado por Santiago) de los casos de
Deudas que el equipo no pudo probar o informó con una observación:
CP-DEU-039, 043 a 048, 049C, 050 a 050D, 057, 063, 069B, 070, 071 y 072 a 093.
43 PASSED y 1 FAILED (CP-DEU-063, DEF-037: el primer clic en «US$» de
«Nueva deuda» se pierde). Actualiza 04, 05, 06 (md y xlsx) y el README.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega-2/05-reportes-de-defectos.xlsx
+++ b/entrega-2/05-reportes-de-defectos.xlsx
@@ -16,6 +16,7 @@
     <sheet name="DEF-034" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="DEF-035" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="DEF-036" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="DEF-037" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -504,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -856,6 +857,43 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>DEF-037</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>El primer clic en «US$» de «Nueva deuda» se pierde: el error de «Persona» corre los botones y la moneda no se selecciona</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Abierto · se reproduce el 2026-10-27</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>CP-DEU-063</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>US-36 · Cargar una deuda suelta (CA-6, FR-18)</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>sin issue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
@@ -868,7 +906,188 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId8"/>
   </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31.83" customWidth="1" min="1" max="1"/>
+    <col width="63.66" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="45" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>[DEF-037] El primer clic en «US$» de «Nueva deuda» se pierde: el error de «Persona» corre los botones y la moneda no se selecciona</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Description / Overview</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>En «Nueva deuda», si el primer clic sobre el formulario es en «US$», la moneda no se selecciona y no aparece el campo «Tipo de cambio (ARS por US$)». Hace falta un segundo clic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Reproduction Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>1- Abrir la app e iniciar sesión con un usuario de prueba (con la configuración inicial salteada).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>2- Abrir /debts/new (Deudas → «Nueva deuda»): el foco queda en «Persona».</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>3- Sin escribir nada, hacer clic en «US$».</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>4- Mirar el formulario: la moneda sigue sin cambiar, no aparece el campo «Tipo de cambio (ARS por US$)» y debajo de «Persona» aparece «Ingresá el nombre de la persona».</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>5- Hacer clic otra vez en «US$»: ahora sí se selecciona y aparece el campo «Tipo de cambio».</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Expected Behavior</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>CP-DEU-063 (paso 6): al hacer clic en «US$» se selecciona la moneda y aparece el campo «Tipo de cambio (ARS por US$)».</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Actual Behavior</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>El primer clic en «US$» no hace nada visible. Al salir del foco de «Persona» aparece el error «Ingresá el nombre de la persona» y los botones bajan unos 26 px (la caja de «US$» pasa de y = 343,8 a y = 370,0 entre apretar y soltar el botón del mouse), así que el clic cae en otro elemento. El segundo clic funciona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Incidence / Severity / Probability of reproduction</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Severidad Media - no se pierden datos y con un segundo clic se puede seguir, pero quien carga una deuda en dólares piensa que la moneda no funciona o que falta el campo del tipo de cambio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>100 % (3 de 3 ejecuciones).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Story and Acceptance Criteria affected</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>US-36 · CA-6: cargar una deuda suelta en US$ con tipo de cambio (CP-DEU-063, paso 6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Browsers tested</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Chromium (Playwright 1.63), ventana de 420 × 900. No se probó en otros navegadores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="225" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>- Defect ID: DEF-037
+- Estado: Abierto · se reproduce el 2026-10-27
+- Issue de GitHub: sin issue
+- Caso de prueba: CP-DEU-063
+- Encontrado en: ejecución de CP-DEU-063 (Entrega 2).
+- Reportó: Claude Code (IA), supervisado por Santiago
+- Evidencia: Medidas de la corrida de CP-DEU-063 (posición de «US$» antes y después de apretar el mouse)
+- Causa probable: la validación al perder el foco muestra el mensaje de error entre el mousedown y el mouseup y desplaza los botones, de modo que el clic no llega al botón. No se corrigió nada. Con un segundo clic el resto del caso se cumple (≈ $0,01 y se guarda amount 0.01, fx_rate 0.5000 y amount_ars 0.01). Puede explicar parte de las dudas del equipo sobre los casos de tipo de cambio en US$ (CP-DEU-050C y 050D).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1086,7 +1305,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1099,7 +1317,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1140,7 +1357,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -1153,7 +1369,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="60" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -1166,7 +1381,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
@@ -1186,7 +1400,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="60" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
@@ -1199,7 +1412,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -1212,7 +1424,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
@@ -1225,7 +1436,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24" ht="240" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
@@ -1275,7 +1485,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1288,7 +1497,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1329,7 +1537,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -1342,7 +1549,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -1355,7 +1561,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
@@ -1375,7 +1580,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
@@ -1388,7 +1592,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -1401,7 +1604,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
@@ -1414,7 +1616,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24" ht="240" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
@@ -1464,7 +1665,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1477,7 +1677,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1518,7 +1717,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -1531,7 +1729,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -1544,7 +1741,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
@@ -1564,7 +1760,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
@@ -1577,7 +1772,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -1590,7 +1784,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
@@ -1603,7 +1796,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24" ht="180" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
@@ -1653,7 +1845,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="75" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1666,7 +1857,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1700,7 +1890,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
@@ -1713,7 +1902,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -1726,7 +1914,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
@@ -1746,7 +1933,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
@@ -1759,7 +1945,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
@@ -1772,7 +1957,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
@@ -1785,7 +1969,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="165" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
@@ -1835,7 +2018,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="75" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1848,7 +2030,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1882,7 +2063,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
@@ -1895,7 +2075,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -1908,7 +2087,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
@@ -1928,7 +2106,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
@@ -1941,7 +2118,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
@@ -1954,7 +2130,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
@@ -1967,7 +2142,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="225" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
@@ -2017,7 +2191,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -2030,7 +2203,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -2050,7 +2222,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
@@ -2063,7 +2234,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
@@ -2076,7 +2246,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -2096,7 +2265,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
@@ -2109,7 +2277,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
@@ -2122,7 +2289,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19" ht="45" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
@@ -2135,7 +2301,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21" ht="210" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
@@ -2185,7 +2350,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -2198,7 +2362,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -2225,7 +2388,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
@@ -2238,7 +2400,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -2251,7 +2412,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -2271,7 +2431,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
@@ -2284,7 +2443,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
@@ -2297,7 +2455,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="45" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -2310,7 +2467,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="165" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(entrega-2): recorta el catálogo de V2 de 672 a 206 casos y lo renumera
El catálogo era demasiado largo para revisarlo en la materia: se quitaron
los casos que repetían una regla con otro valor (testids por pantalla y
ancho, bordes repetidos, pares UI/API de cada campo), los de funciones sin
implementar (US-80, US-81, US-82 salvo tres casos, US-83) y los que estaban
en DUDA por errores del caso.

Quedan NAV 25, DEU 61, EXP 31, SUS 48 e IMP 41, con IDs consecutivos desde
001 en cada módulo. Se actualizan casos, especificación, ejecución,
defectos, reporte, README y los cuatro Excel (189 casos con resultado:
178 PASSED, 8 FAILED, 3 BLOCKED). Se retira DEF-029, que era un error del
caso. La tabla equivalencia-ids.md relaciona cada ID anterior con el nuevo.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega-2/05-reportes-de-defectos.xlsx
+++ b/entrega-2/05-reportes-de-defectos.xlsx
@@ -8,15 +8,14 @@
   </bookViews>
   <sheets>
     <sheet name="Index" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="DEF-029" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="DEF-030" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DEF-031" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="DEF-032" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="DEF-033" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="DEF-034" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="DEF-035" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="DEF-036" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="DEF-037" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="DEF-030" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="DEF-031" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="DEF-032" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="DEF-033" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="DEF-034" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="DEF-035" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="DEF-036" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="DEF-037" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -562,51 +561,51 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>DEF-029</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>La baja de un gasto (delete_transaction) responde 204 sin cuerpo y el caso espera 200 con null</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Abierto · se reproduce el 2026-10-25</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>CP-NAV-084</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>US-70 · Reintento sin duplicar al recuperar un gasto (CA-21)</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>— (sin issue)</t>
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>DEF-030</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Tocar fuera de la hoja «Exportar movimientos» no la cierra</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Abierto · se reproduce el 2026-10-27</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>CP-EXP-027</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>US-47 · Exportar movimientos a CSV (CA-23)</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>sin issue</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>DEF-030</t>
+          <t>DEF-031</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Tocar fuera de la hoja «Exportar movimientos» no la cierra</t>
+          <t>«Atrás» y «Adelante» del navegador cambian la URL pero la hoja de exportar queda abierta</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -621,12 +620,12 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>CP-EXP-062 (también quita valor a CP-EXP-070)</t>
+          <t>CP-EXP-028 (el caso equivalente con «Adelante» se recortó del catálogo el 2026-10-27)</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>US-47 · Exportar movimientos a CSV (CA-23)</t>
+          <t>US-47 · Exportar movimientos a CSV (CA-24 y requisito «todo cambio de URL»)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -638,12 +637,12 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>DEF-031</t>
+          <t>DEF-032</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>«Atrás» y «Adelante» del navegador cambian la URL pero la hoja de exportar queda abierta</t>
+          <t>«Atrás» durante «Exportando…» no cancela la exportación: el archivo se descarga igual</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -658,12 +657,12 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>CP-EXP-063 y CP-EXP-065</t>
+          <t>CP-EXP-029</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>US-47 · Exportar movimientos a CSV (CA-24 y requisito «todo cambio de URL»)</t>
+          <t>US-47 · Exportar movimientos a CSV (CA-24)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -675,17 +674,17 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>DEF-032</t>
+          <t>DEF-033</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>«Atrás» durante «Exportando…» no cancela la exportación: el archivo se descarga igual</t>
+          <t>La tarjeta de una fila lista muestra la categoría y la cuenta como están escritas en el archivo, no como se llaman en Biyu</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -695,12 +694,12 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>CP-EXP-064</t>
+          <t>CP-IMP-024</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>US-47 · Exportar movimientos a CSV (CA-24)</t>
+          <t>US-76 · Revisión de filas (CA-5)</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -712,12 +711,12 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>DEF-033</t>
+          <t>DEF-034</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>La tarjeta de una fila lista muestra la categoría y la cuenta como están escritas en el archivo, no como se llaman en Biyu</t>
+          <t>Operar sobre la suscripción de otro usuario responde HTTP 500 en lugar de 404</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -732,12 +731,12 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>CP-IMP-052</t>
+          <t>CP-SUS-032 (otros tres casos con el mismo defecto se recortaron del catálogo el 2026-10-27)</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>US-76 · Revisión de filas (CA-5)</t>
+          <t>US-56 · CA-9, US-57 · CA-7, US-58 · CA-9 y US-59 (Pausar, reanudar, cancelar y editar: par de autorización)</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -749,12 +748,12 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>DEF-034</t>
+          <t>DEF-035</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Operar sobre la suscripción de otro usuario responde HTTP 500 en lugar de 404</t>
+          <t>Sin sesión, la API responde HTTP 401 y los casos esperan 403</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -769,12 +768,12 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>CP-SUS-094, CP-SUS-100, CP-SUS-107 y CP-SUS-129</t>
+          <t>CP-SUS-022 (otros cinco casos con el mismo defecto se recortaron del catálogo el 2026-10-27)</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>US-56 · CA-9, US-57 · CA-7, US-58 · CA-9 y US-59 (Pausar, reanudar, cancelar y editar: par de autorización)</t>
+          <t>US-52 · CA-13 y US-56 · CA-9, US-57 · CA-7, US-58 · CA-9, US-59 (rol anon)</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -786,12 +785,12 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>DEF-035</t>
+          <t>DEF-036</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Sin sesión, la API responde HTTP 401 y los casos esperan 403</t>
+          <t>La vista previa del calendario no marca con data-blocked="false" las filas que no están bloqueadas</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -806,12 +805,12 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>CP-SUS-065, CP-SUS-066, CP-SUS-095, CP-SUS-101, CP-SUS-108 y CP-SUS-130</t>
+          <t>CP-SUS-048</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>US-52 · CA-13 y US-56 · CA-9, US-57 · CA-7, US-58 · CA-9, US-59 (rol anon)</t>
+          <t>US-61 · Vista previa del calendario al dar de alta una suscripción</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -823,17 +822,17 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>DEF-036</t>
+          <t>DEF-037</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>La vista previa del calendario no marca con data-blocked="false" las filas que no están bloqueadas</t>
+          <t>El primer clic en «US$» de «Nueva deuda» se pierde: el error de «Persona» corre los botones y la moneda no se selecciona</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -843,12 +842,12 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>CP-SUS-157</t>
+          <t>CP-DEU-024</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>US-61 · Vista previa del calendario al dar de alta una suscripción</t>
+          <t>US-36 · Cargar una deuda suelta (CA-6, FR-18)</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -858,39 +857,9 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>DEF-037</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>El primer clic en «US$» de «Nueva deuda» se pierde: el error de «Persona» corre los botones y la moneda no se selecciona</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>Abierto · se reproduce el 2026-10-27</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>CP-DEU-063</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>US-36 · Cargar una deuda suelta (CA-6, FR-18)</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>sin issue</t>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>#'DEF-037'!A1</t>
         </is>
       </c>
     </row>
@@ -912,7 +881,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -925,7 +894,7 @@
     <col width="63.66" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="45" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Title</t>
@@ -933,11 +902,11 @@
       </c>
       <c r="B1" s="9" t="inlineStr">
         <is>
-          <t>[DEF-037] El primer clic en «US$» de «Nueva deuda» se pierde: el error de «Persona» corre los botones y la moneda no se selecciona</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="45" customHeight="1">
+          <t>[DEF-030] Tocar fuera de la hoja «Exportar movimientos» no la cierra</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Description / Overview</t>
@@ -945,11 +914,11 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>En «Nueva deuda», si el primer clic sobre el formulario es en «US$», la moneda no se selecciona y no aparece el campo «Tipo de cambio (ARS por US$)». Hace falta un segundo clic.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
+          <t>Tocar fuera de la hoja «Exportar movimientos» no la cierra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="45" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -957,39 +926,39 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>1- Abrir la app e iniciar sesión con un usuario de prueba (con la configuración inicial salteada).</t>
+          <t>1- Abrir la app e iniciar sesión con un usuario de prueba. Si aparece la configuración inicial, tocar «Saltear» en sus 4 pasos.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>2- Abrir /debts/new (Deudas → «Nueva deuda»): el foco queda en «Persona».</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1">
+          <t>2- Crear un gasto con fecha en septiembre de 2026 y abrir en el navegador /transactions?period=2026-09.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>3- Sin escribir nada, hacer clic en «US$».</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
+          <t>3- Tocar «Exportar» arriba a la derecha: se abre la hoja «Exportar movimientos».</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>4- Mirar el formulario: la moneda sigue sin cambiar, no aparece el campo «Tipo de cambio (ARS por US$)» y debajo de «Persona» aparece «Ingresá el nombre de la persona».</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
+          <t>4- Hacer clic sobre el fondo oscuro, fuera de la hoja (por ejemplo, en la esquina superior izquierda de la pantalla).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>5- Hacer clic otra vez en «US$»: ahora sí se selecciona y aparece el campo «Tipo de cambio».</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
+          <t>5- Mirar si la hoja sigue abierta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Expected Behavior</t>
@@ -997,11 +966,11 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>CP-DEU-063 (paso 6): al hacer clic en «US$» se selecciona la moneda y aparece el campo «Tipo de cambio (ARS por US$)».</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="90" customHeight="1">
+          <t>CA-23 / CP-EXP-027: tocar fuera de la hoja la cierra sin descargar nada y la URL conserva ?period=2026-09 (mientras no esté en «Exportando…»).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="60" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Actual Behavior</t>
@@ -1009,11 +978,11 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>El primer clic en «US$» no hace nada visible. Al salir del foco de «Persona» aparece el error «Ingresá el nombre de la persona» y los botones bajan unos 26 px (la caja de «US$» pasa de y = 343,8 a y = 370,0 entre apretar y soltar el botón del mouse), así que el clic cae en otro elemento. El segundo clic funciona.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="60" customHeight="1">
+          <t>La hoja sigue abierta. El elemento que recibe el clic en esa posición es el div de fondo (clases fixed inset-0 -z-10, aria-hidden="true"), no el contenedor de la hoja. Solo «Cancelar» y Escape la cierran.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Incidence / Severity / Probability of reproduction</t>
@@ -1021,7 +990,7 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Severidad Media - no se pierden datos y con un segundo clic se puede seguir, pero quien carga una deuda en dólares piensa que la moneda no funciona o que falta el campo del tipo de cambio.</t>
+          <t>Severidad Media - no se pierden datos y la hoja se puede cerrar con «Cancelar» o Escape, pero se incumple CA-23 y un gesto habitual no hace nada.</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1001,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1">
+    <row r="18" ht="60" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Story and Acceptance Criteria affected</t>
@@ -1040,7 +1009,7 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>US-36 · CA-6: cargar una deuda suelta en US$ con tipo de cambio (CP-DEU-063, paso 6).</t>
+          <t>US-47 · CA-23: «Tocar fuera de la hoja la cierra sin descargar» (CP-EXP-027). Además, el caso «tocar fuera no cierra la hoja durante Exportando», recortado del catálogo, pasaba sin probar nada mientras este defecto siguiera abierto.</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1025,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="30" customHeight="1">
+    <row r="22" ht="45" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Environment</t>
@@ -1064,11 +1033,11 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="225" customHeight="1">
+          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63), reloj fijado en 09/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="240" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>Notes</t>
@@ -1076,202 +1045,14 @@
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>- Defect ID: DEF-037
+          <t>- Defect ID: DEF-030
 - Estado: Abierto · se reproduce el 2026-10-27
 - Issue de GitHub: sin issue
-- Caso de prueba: CP-DEU-063
-- Encontrado en: ejecución de CP-DEU-063 (Entrega 2).
+- Caso de prueba: CP-EXP-027
+- Encontrado en: ejecución de CP-EXP-027 (Entrega 2).
 - Reportó: Claude Code (IA), supervisado por Santiago
-- Evidencia: Medidas de la corrida de CP-DEU-063 (posición de «US$» antes y después de apretar el mouse)
-- Causa probable: la validación al perder el foco muestra el mensaje de error entre el mousedown y el mouseup y desplaza los botones, de modo que el clic no llega al botón. No se corrigió nada. Con un segundo clic el resto del caso se cumple (≈ $0,01 y se guarda amount 0.01, fx_rate 0.5000 y amount_ars 0.01). Puede explicar parte de las dudas del equipo sobre los casos de tipo de cambio en US$ (CP-DEU-050C y 050D).</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="31.8" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>[DEF-029] La baja de un gasto (delete_transaction) responde 204 sin cuerpo y el caso espera 200 con null</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="49" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Description / Overview</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Al eliminar un gasto llamando a la función delete_transaction, el sistema responde HTTP 204 sin cuerpo. El caso CP-NAV-084 espera HTTP 200 con el cuerpo null. La baja en sí funciona bien (el gasto queda eliminado y su cuota histórica se conserva); lo que no coincide es la respuesta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Reproduction Steps</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>1- Versión donde ocurre: main en f096e22 (app local contra Supabase local con todas las migraciones aplicadas).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="34" customHeight="1">
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>2- Tener un usuario de prueba con la cuenta «Visa BBVA» y la categoría «Comida» (ver los pre-requisitos de CP-NAV-084) y su token de sesión.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="94" customHeight="1">
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>3- En Postman, enviar un POST a SUPABASE_URL/rest/v1/rpc/create_transaction con los encabezados apikey, Authorization (Bearer + token) y Content-Type: application/json, y el cuerpo {"p_type":"expense","p_amount":"12500.00","p_currency":"ARS","p_fx_rate":null,"p_category_id":"&lt;id de Comida&gt;","p_account_id":"&lt;id de Visa BBVA&gt;","p_installments_count":1,"p_occurred_on":"2026-10-06","p_description":"Almuerzo","p_shared_person":null,"p_shared_amount":null,"p_request_id":"84000000-0000-4000-8000-000000000084"}. Anotar el identificador que devuelve (ID-1).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>4- Enviar un POST a SUPABASE_URL/rest/v1/rpc/delete_transaction con los mismos encabezados y el cuerpo {"p_transaction_id":"&lt;ID-1&gt;"}.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="19" customHeight="1">
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>5- Mirar el código de respuesta y si trae cuerpo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>6- Enviar un GET a SUPABASE_URL/rest/v1/transactions?select=id,request_id,deleted_at&amp;request_id=eq.84000000-0000-4000-8000-000000000084 y comprobar la fila.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Expected Behavior</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Según el caso CP-NAV-084 (paso 2): HTTP 200 y el cuerpo JSON null.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Actual Behavior</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>HTTP 204 (sin contenido) y cuerpo vacío. La fila de la transacción queda con deleted_at con fecha y la cuota histórica se conserva.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Incidence / Severity / Probability of reproduction</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Severidad Baja: la baja lógica y la cuota histórica se comportan bien; solo difiere el código de respuesta del contrato que espera el caso, y no afecta a lo que ve el usuario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="19" customHeight="1">
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>100 % (1 de 1 ejecución).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="49" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Story and Acceptance Criteria affected</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>US-70 · CA-21: «Recuperar un gasto ya guardado y eliminado no crea otro gasto». El criterio funcional se cumple; el caso CP-NAV-084 pide además un código de respuesta que la función no devuelve.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Browsers tested</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>No aplica: llamada directa a la API (Postman).</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="32" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Environment</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>Local: Vite (http://127.0.0.1:5173) + Supabase local · main f096e22 · migraciones hasta 20261012000000.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="230" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>- Defect ID: DEF-029
-- Estado: Abierto · se reproduce el 2026-10-25
-- Issue de GitHub: sin issue
-- Caso de prueba: CP-NAV-084
-- Encontrado en: ejecución de CP-NAV-084 (Entrega 2).
-- Reportó: Claude Code, supervisado por Santiago
-- Causa probable: la función delete_transaction está definida como «returns void» (supabase/migrations/20260927180000_delete_transaction_rpc.sql) y PostgREST responde 204 No Content a las funciones que no devuelven nada. Parece un error del resultado esperado del caso y no de la aplicación.
-- Decisión pendiente: corregir el caso (esperar 204) o cambiar la función para que devuelva un valor. Por decisión de Santiago no se corrigió nada.
-- Evidencia: respuesta 204 de delete_transaction y consulta de la fila con deleted_at con fecha (ver CP-NAV-084 en 04-ejecucion).</t>
+- Evidencia: Observado en la corrida de CP-EXP-027: la hoja sigue abierta tras el clic; document.elementFromPoint(5, 5) = DIV.fixed.inset-0.-z-10.bg-[rgba(43,30,25,0.32)], aria-hidden=true
+- Causa probable: en src/components/transactions/ExportTransactionsDialog.tsx el cierre por clic exige e.target === e.currentTarget, pero el div de fondo es hijo del contenedor y cubre toda la pantalla: recibe el clic y el destino nunca coincide. No se corrigió nada.</t>
         </is>
       </c>
     </row>
@@ -1301,11 +1082,11 @@
       </c>
       <c r="B1" s="9" t="inlineStr">
         <is>
-          <t>[DEF-030] Tocar fuera de la hoja «Exportar movimientos» no la cierra</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1">
+          <t>[DEF-031] «Atrás» y «Adelante» del navegador cambian la URL pero la hoja de exportar queda abierta</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Description / Overview</t>
@@ -1313,11 +1094,11 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Tocar fuera de la hoja «Exportar movimientos» no la cierra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="45" customHeight="1">
+          <t>Con la hoja «Exportar movimientos» abierta, «Atrás» y «Adelante» del navegador cambian el período de la URL pero la hoja no se cierra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -1325,35 +1106,35 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>1- Abrir la app e iniciar sesión con un usuario de prueba. Si aparece la configuración inicial, tocar «Saltear» en sus 4 pasos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
+          <t>1- Abrir la app e iniciar sesión con un usuario de prueba (con la configuración inicial salteada).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1">
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>2- Crear un gasto con fecha en septiembre de 2026 y abrir en el navegador /transactions?period=2026-09.</t>
+          <t>2- Abrir en el navegador /transactions?period=2026-08.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>3- Tocar «Exportar» arriba a la derecha: se abre la hoja «Exportar movimientos».</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
+          <t>3- Tocar el botón de mes siguiente: la URL pasa a ?period=2026-09.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>4- Hacer clic sobre el fondo oscuro, fuera de la hoja (por ejemplo, en la esquina superior izquierda de la pantalla).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1">
+          <t>4- Tocar «Exportar»: se abre la hoja.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>5- Mirar si la hoja sigue abierta.</t>
+          <t>5- Hacer clic en «Atrás» del navegador y mirar la URL y la hoja. (Para el caso equivalente con «Adelante», recortado: abrir la hoja en agosto, después de haber vuelto desde septiembre, y hacer clic en «Adelante».)</t>
         </is>
       </c>
     </row>
@@ -1365,11 +1146,11 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>CA-23 / CP-EXP-062: tocar fuera de la hoja la cierra sin descargar nada y la URL conserva ?period=2026-09 (mientras no esté en «Exportando…»).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="60" customHeight="1">
+          <t>CA-24 / CP-EXP-028 y su caso equivalente con «Adelante»: la hoja se cierra, la URL pasa a ?period=2026-08 (con «Adelante», a ?period=2026-09) y no se descarga archivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Actual Behavior</t>
@@ -1377,7 +1158,7 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>La hoja sigue abierta. El elemento que recibe el clic en esa posición es el div de fondo (clases fixed inset-0 -z-10, aria-hidden="true"), no el contenedor de la hoja. Solo «Cancelar» y Escape la cierran.</t>
+          <t>La URL cambia al período anterior (o al siguiente) y la hoja sigue abierta. El evento popstate sí se dispara (verificado en 3 de 3 repeticiones), pero la hoja no se cierra.</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1170,7 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Severidad Media - no se pierden datos y la hoja se puede cerrar con «Cancelar» o Escape, pero se incumple CA-23 y un gesto habitual no hace nada.</t>
+          <t>Severidad Media - no se pierden ni se duplican datos, pero la hoja queda sobre otro período y el usuario puede descargar un mes distinto del que ve en la URL.</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1181,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="60" customHeight="1">
+    <row r="18" ht="45" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Story and Acceptance Criteria affected</t>
@@ -1408,7 +1189,7 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>US-47 · CA-23: «Tocar fuera de la hoja la cierra sin descargar» (CP-EXP-062). Además, CP-EXP-070 («tocar fuera no cierra la hoja durante Exportando») pasa sin probar nada mientras este defecto siga abierto.</t>
+          <t>US-47 · CA-24: «Si cambia la URL o se presiona Atrás, la hoja se cierra y no se descarga nada», y el requisito «todo cambio de URL cierra la hoja» (CP-EXP-028 y su caso equivalente con «Adelante», recortado).</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1201,7 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Chromium (Playwright 1.63), ventana de 420 × 900. No se probó en otros navegadores.</t>
+          <t>Chromium (Playwright 1.63). No se probó en otros navegadores.</t>
         </is>
       </c>
     </row>
@@ -1444,14 +1225,14 @@
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>- Defect ID: DEF-030
+          <t>- Defect ID: DEF-031
 - Estado: Abierto · se reproduce el 2026-10-27
 - Issue de GitHub: sin issue
-- Caso de prueba: CP-EXP-062 (también quita valor a CP-EXP-070)
-- Encontrado en: ejecución de CP-EXP-062 (Entrega 2).
+- Caso de prueba: CP-EXP-028 (el caso equivalente con «Adelante» se recortó del catálogo el 2026-10-27)
+- Encontrado en: ejecución de CP-EXP-028 y de su caso equivalente con «Adelante» (Entrega 2).
 - Reportó: Claude Code (IA), supervisado por Santiago
-- Evidencia: Observado en la corrida de CP-EXP-062: la hoja sigue abierta tras el clic; document.elementFromPoint(5, 5) = DIV.fixed.inset-0.-z-10.bg-[rgba(43,30,25,0.32)], aria-hidden=true
-- Causa probable: en src/components/transactions/ExportTransactionsDialog.tsx el cierre por clic exige e.target === e.currentTarget, pero el div de fondo es hijo del contenedor y cubre toda la pantalla: recibe el clic y el destino nunca coincide. No se corrigió nada.</t>
+- Evidencia: Observado en las corridas de CP-EXP-028 (y su caso equivalente con «Adelante», recortado): URL cambiada con la hoja abierta; log de popstate: ['popstate@?period=2026-08']
+- Causa no determinada. En ExportTransactionsDialog.tsx hay un efecto que cierra la hoja cuando cambia location.key y un oyente de popstate; ninguno logra cerrarla. Hipótesis sin confirmar: el efecto que reinicia initialLocationKeyRef cuando cambia location.key corre antes del que compara la clave y la deja siempre igual. No se corrigió nada.</t>
         </is>
       </c>
     </row>
@@ -1481,11 +1262,11 @@
       </c>
       <c r="B1" s="9" t="inlineStr">
         <is>
-          <t>[DEF-031] «Atrás» y «Adelante» del navegador cambian la URL pero la hoja de exportar queda abierta</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="45" customHeight="1">
+          <t>[DEF-032] «Atrás» durante «Exportando…» no cancela la exportación: el archivo se descarga igual</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Description / Overview</t>
@@ -1493,7 +1274,7 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Con la hoja «Exportar movimientos» abierta, «Atrás» y «Adelante» del navegador cambian el período de la URL pero la hoja no se cierra.</t>
+          <t>«Atrás» durante «Exportando…» no cancela la exportación: el archivo se descarga igual.</t>
         </is>
       </c>
     </row>
@@ -1505,39 +1286,39 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>1- Abrir la app e iniciar sesión con un usuario de prueba (con la configuración inicial salteada).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1">
+          <t>1- Abrir la app e iniciar sesión con un usuario de prueba que tenga un gasto de septiembre de 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>2- Abrir en el navegador /transactions?period=2026-08.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
+          <t>2- Abrir /transactions?period=2026-08, tocar el mes siguiente (URL ?period=2026-09) y tocar «Exportar».</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>3- Tocar el botón de mes siguiente: la URL pasa a ?period=2026-09.</t>
+          <t>3- Demorar unos segundos las respuestas de /rest/v1/transactions (en las pruebas, 3 s con Playwright; en DevTools, «1 kbit/s» y latencia 2000 ms).</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>4- Tocar «Exportar»: se abre la hoja.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="45" customHeight="1">
+          <t>4- Tocar «Descargar CSV»: el botón pasa a «Exportando…».</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>5- Hacer clic en «Atrás» del navegador y mirar la URL y la hoja. (Para CP-EXP-065: abrir la hoja en agosto, después de haber vuelto desde septiembre, y hacer clic en «Adelante».)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="45" customHeight="1">
+          <t>5- Hacer clic en «Atrás» del navegador y esperar a que termine la demora.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Expected Behavior</t>
@@ -1545,7 +1326,7 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>CA-24 / CP-EXP-063 y 065: la hoja se cierra, la URL pasa a ?period=2026-08 (con «Adelante», a ?period=2026-09) y no se descarga archivo.</t>
+          <t>CA-24 / CP-EXP-029 (paso 22): la exportación se cancela; no aparece ningún archivo ni aviso de éxito.</t>
         </is>
       </c>
     </row>
@@ -1557,11 +1338,11 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>La URL cambia al período anterior (o al siguiente) y la hoja sigue abierta. El evento popstate sí se dispara (verificado en 3 de 3 repeticiones), pero la hoja no se cierra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="45" customHeight="1">
+          <t>Al terminar la lectura se descarga biyu-movimientos-2026-09.csv y aparece el aviso «Exportamos 1 movimiento» (1 descarga y 1 aviso), con el usuario ya en ?period=2026-08.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Incidence / Severity / Probability of reproduction</t>
@@ -1569,18 +1350,18 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Severidad Media - no se pierden ni se duplican datos, pero la hoja queda sobre otro período y el usuario puede descargar un mes distinto del que ve en la URL.</t>
+          <t>Severidad Media - se descarga un archivo que el usuario ya había abandonado; no afecta datos guardados.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>100 % (3 de 3 ejecuciones).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="45" customHeight="1">
+          <t>100 % (2 de 2 ejecuciones).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Story and Acceptance Criteria affected</t>
@@ -1588,7 +1369,7 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>US-47 · CA-24: «Si cambia la URL o se presiona Atrás, la hoja se cierra y no se descarga nada», y el requisito «todo cambio de URL cierra la hoja» (CP-EXP-063 y CP-EXP-065).</t>
+          <t>US-47 · CA-24: «Atrás durante Exportando… cancela la descarga» (CP-EXP-029).</t>
         </is>
       </c>
     </row>
@@ -1616,7 +1397,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="240" customHeight="1">
+    <row r="24" ht="180" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>Notes</t>
@@ -1624,14 +1405,14 @@
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>- Defect ID: DEF-031
+          <t>- Defect ID: DEF-032
 - Estado: Abierto · se reproduce el 2026-10-27
 - Issue de GitHub: sin issue
-- Caso de prueba: CP-EXP-063 y CP-EXP-065
-- Encontrado en: ejecución de CP-EXP-063 y CP-EXP-065 (Entrega 2).
+- Caso de prueba: CP-EXP-029
+- Encontrado en: ejecución de CP-EXP-029 (Entrega 2).
 - Reportó: Claude Code (IA), supervisado por Santiago
-- Evidencia: Observado en las corridas de CP-EXP-063 y CP-EXP-065: URL cambiada con la hoja abierta; log de popstate: ['popstate@?period=2026-08']
-- Causa no determinada. En ExportTransactionsDialog.tsx hay un efecto que cierra la hoja cuando cambia location.key y un oyente de popstate; ninguno logra cerrarla. Hipótesis sin confirmar: el efecto que reinicia initialLocationKeyRef cuando cambia location.key corre antes del que compara la clave y la deja siempre igual. No se corrigió nada.</t>
+- Evidencia: Observado en la corrida de CP-EXP-029: aviso de éxito en el período anterior; descargas registradas por el navegador = 1
+- Relacionado con DEF-031: el cierre por «Atrás» no llega a abortar la exportación en curso (AbortController). No se investigó a fondo. No se corrigió nada.</t>
         </is>
       </c>
     </row>
@@ -1646,14 +1427,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.83" customWidth="1" min="1" max="1"/>
     <col width="63.66" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="45" customHeight="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Title</t>
@@ -1661,11 +1442,11 @@
       </c>
       <c r="B1" s="9" t="inlineStr">
         <is>
-          <t>[DEF-032] «Atrás» durante «Exportando…» no cancela la exportación: el archivo se descarga igual</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
+          <t>[DEF-033] La tarjeta de una fila lista muestra la categoría y la cuenta como están escritas en el archivo, no como se llaman en Biyu</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="75" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Description / Overview</t>
@@ -1673,11 +1454,11 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>«Atrás» durante «Exportando…» no cancela la exportación: el archivo se descarga igual.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
+          <t>En la Revisión del importador, la tarjeta de una fila «Lista» muestra el texto de la categoría y de la cuenta tal cual está en el Excel (por ejemplo «educación» y «efectivo»), en lugar del nombre con el que existen en Biyu («Educación» y «Efectivo»).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="45" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -1685,133 +1466,126 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>1- Abrir la app e iniciar sesión con un usuario de prueba que tenga un gasto de septiembre de 2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
+          <t>1- Abrir la app e iniciar sesión con un usuario de prueba (con la configuración inicial salteada) y tocar «Importar desde Excel».</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>2- Abrir /transactions?period=2026-08, tocar el mes siguiente (URL ?period=2026-09) y tocar «Exportar».</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
+          <t>2- Armar un .xlsx con los encabezados de la plantilla y una fila: fecha 01/09/2026, Tipo « gasto » (con espacios), Monto 10, Moneda «usd», Tipo de cambio 1450, Categoría «  educación  », Cuenta «  efectivo  », Cuotas 1, Nota «Coincidencia».</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>3- Demorar unos segundos las respuestas de /rest/v1/transactions (en las pruebas, 3 s con Playwright; en DevTools, «1 kbit/s» y latencia 2000 ms).</t>
+          <t>3- Tocar «Elegir archivo .xlsx» y elegir el archivo.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>4- Tocar «Descargar CSV»: el botón pasa a «Exportando…».</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>5- Hacer clic en «Atrás» del navegador y esperar a que termine la demora.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
+          <t>4- Mirar la tarjeta «Fila 2» de la Revisión.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Expected Behavior</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
-        <is>
-          <t>CA-24 / CP-EXP-064 (paso 22): la exportación se cancela; no aparece ningún archivo ni aviso de éxito.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>CP-IMP-024 (paso 10): «Fila 2» está «Lista» y muestra «Gasto», «US$10,00», «Educación», «Efectivo» y «TC 1.450,00».</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Actual Behavior</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
-        <is>
-          <t>Al terminar la lectura se descarga biyu-movimientos-2026-09.csv y aparece el aviso «Exportamos 1 movimiento» (1 descarga y 1 aviso), con el usuario ya en ?period=2026-08.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>La fila está «Lista» (la coincidencia sin distinguir mayúsculas ni espacios funciona) pero la tarjeta dice «01/09/2026 · Gasto · educación · efectivo · TC 1.450,00 US$10,00»: muestra el texto del archivo, no los nombres de Biyu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Incidence / Severity / Probability of reproduction</t>
         </is>
       </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Severidad Baja - las filas se importan bien (se asocian a la categoría y cuenta correctas); solo cambia lo que se muestra antes de confirmar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1">
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Severidad Media - se descarga un archivo que el usuario ya había abandonado; no afecta datos guardados.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t>100 % (2 de 2 ejecuciones).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="8" t="inlineStr">
+          <t>100 % (1 de 1 ejecución).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>Story and Acceptance Criteria affected</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>US-47 · CA-24: «Atrás durante Exportando… cancela la descarga» (CP-EXP-064).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>US-76 · CA-5: coincidencia de nombres sin distinguir mayúsculas ni espacios, con la tarjeta mostrando los nombres de Biyu (CP-IMP-024).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Browsers tested</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Chromium (Playwright 1.63). No se probó en otros navegadores.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="45" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63), reloj fijado en 09/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="180" customHeight="1">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="165" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B24" s="11" t="inlineStr">
-        <is>
-          <t>- Defect ID: DEF-032
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>- Defect ID: DEF-033
 - Estado: Abierto · se reproduce el 2026-10-27
 - Issue de GitHub: sin issue
-- Caso de prueba: CP-EXP-064
-- Encontrado en: ejecución de CP-EXP-064 (Entrega 2).
+- Caso de prueba: CP-IMP-024
+- Encontrado en: ejecución de CP-IMP-024 (Entrega 2).
 - Reportó: Claude Code (IA), supervisado por Santiago
-- Evidencia: Observado en la corrida de CP-EXP-064: aviso de éxito en el período anterior; descargas registradas por el navegador = 1
-- Relacionado con DEF-031: el cierre por «Atrás» no llega a abortar la exportación en curso (AbortController). No se investigó a fondo. No se corrigió nada.</t>
+- Evidencia: Texto de la tarjeta import-row-2 en la corrida de CP-IMP-024
+- Causa probable: la tarjeta arma el detalle con el texto leído del archivo y no con el nombre del catálogo que resolvió la fila. No se investigó a fondo ni se corrigió nada.</t>
         </is>
       </c>
     </row>
@@ -1833,7 +1607,7 @@
     <col width="63.66" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="45" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Title</t>
@@ -1841,7 +1615,7 @@
       </c>
       <c r="B1" s="9" t="inlineStr">
         <is>
-          <t>[DEF-033] La tarjeta de una fila lista muestra la categoría y la cuenta como están escritas en el archivo, no como se llaman en Biyu</t>
+          <t>[DEF-034] Operar sobre la suscripción de otro usuario responde HTTP 500 en lugar de 404</t>
         </is>
       </c>
     </row>
@@ -1853,11 +1627,11 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>En la Revisión del importador, la tarjeta de una fila «Lista» muestra el texto de la categoría y de la cuenta tal cual está en el Excel (por ejemplo «educación» y «efectivo»), en lugar del nombre con el que existen en Biyu («Educación» y «Efectivo»).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="45" customHeight="1">
+          <t>Cuando un usuario llama a pause_subscription, resume_subscription, cancel_subscription o update_subscription con el identificador de una suscripción de otro usuario, la API rechaza la operación (P0002 «Suscripción no encontrada») pero con HTTP 500 en lugar de 404.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -1865,28 +1639,28 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>1- Abrir la app e iniciar sesión con un usuario de prueba (con la configuración inicial salteada) y tocar «Importar desde Excel».</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="60" customHeight="1">
+          <t>1- Crear dos usuarios de prueba, A y B, con la configuración inicial salteada, y obtener el token de cada uno (PR-04).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>2- Armar un .xlsx con los encabezados de la plantilla y una fila: fecha 01/09/2026, Tipo « gasto » (con espacios), Monto 10, Moneda «usd», Tipo de cambio 1450, Categoría «  educación  », Cuenta «  efectivo  », Cuotas 1, Nota «Coincidencia».</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1">
+          <t>2- Con el token de B, crear una suscripción (POST /rest/v1/rpc/create_subscription) y guardar su id.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>3- Tocar «Elegir archivo .xlsx» y elegir el archivo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1">
+          <t>3- Con el token de A, enviar POST /rest/v1/rpc/pause_subscription con body {"p_subscription_id":"&lt;id de B&gt;"}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>4- Mirar la tarjeta «Fila 2» de la Revisión.</t>
+          <t>4- Mirar el código HTTP y el cuerpo. Repetir con resume_subscription (sobre una pausada), cancel_subscription y update_subscription.</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1672,7 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>CP-IMP-052 (paso 10): «Fila 2» está «Lista» y muestra «Gasto», «US$10,00», «Educación», «Efectivo» y «TC 1.450,00».</t>
+          <t>Los casos esperan HTTP 404 con "code": "P0002" y "message": "Suscripción no encontrada".</t>
         </is>
       </c>
     </row>
@@ -1910,7 +1684,7 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>La fila está «Lista» (la coincidencia sin distinguir mayúsculas ni espacios funciona) pero la tarjeta dice «01/09/2026 · Gasto · educación · efectivo · TC 1.450,00 US$10,00»: muestra el texto del archivo, no los nombres de Biyu.</t>
+          <t>HTTP 500 con {"code":"P0002","details":null,"hint":null,"message":"Suscripción no encontrada"}. El código y el mensaje coinciden; cambia el HTTP. La suscripción de B no se modifica.</t>
         </is>
       </c>
     </row>
@@ -1922,14 +1696,14 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Severidad Baja - las filas se importan bien (se asocian a la categoría y cuenta correctas); solo cambia lo que se muestra antes de confirmar.</t>
+          <t>Severidad Baja - la operación se rechaza bien y no se filtra ningún dato, pero un «no encontrado» se informa como error del servidor.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>100 % (1 de 1 ejecución).</t>
+          <t>100 % (4 de 4 ejecuciones).</t>
         </is>
       </c>
     </row>
@@ -1941,11 +1715,11 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>US-76 · CA-5: coincidencia de nombres sin distinguir mayúsculas ni espacios, con la tarjeta mostrando los nombres de Biyu (CP-IMP-052).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
+          <t>US-56 · CA-9, US-57 · CA-7, US-58 · CA-9: «otro usuario recibe P0002 "Suscripción no encontrada"»; los casos agregan el HTTP 404.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Browsers tested</t>
@@ -1953,11 +1727,11 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Chromium (Playwright 1.63). No se probó en otros navegadores.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
+          <t>No aplica: llamada directa a la API.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="45" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Environment</t>
@@ -1965,11 +1739,11 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="165" customHeight="1">
+          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63) · Edge Functions locales levantadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="225" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Notes</t>
@@ -1977,14 +1751,14 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>- Defect ID: DEF-033
+          <t>- Defect ID: DEF-034
 - Estado: Abierto · se reproduce el 2026-10-27
 - Issue de GitHub: sin issue
-- Caso de prueba: CP-IMP-052
-- Encontrado en: ejecución de CP-IMP-052 (Entrega 2).
+- Caso de prueba: CP-SUS-032 (otros tres casos con el mismo defecto se recortaron del catálogo el 2026-10-27)
+- Encontrado en: ejecución de CP-SUS-032 y de otros tres casos equivalentes (Entrega 2).
 - Reportó: Claude Code (IA), supervisado por Santiago
-- Evidencia: Texto de la tarjeta import-row-2 en la corrida de CP-IMP-052
-- Causa probable: la tarjeta arma el detalle con el texto leído del archivo y no con el nombre del catálogo que resolvió la fila. No se investigó a fondo ni se corrigió nada.</t>
+- Evidencia: Respuesta de la API en las corridas de CP-SUS-032 y de otros tres casos equivalentes
+- Causa probable: PostgREST solo traduce a 4xx algunos códigos de error y P0002 no está entre ellos; hace falta un código propio (por ejemplo PT404) en la función. No se investigó a fondo ni se corrigió nada. Decisión pendiente: cambiar la función o el resultado esperado de los casos.</t>
         </is>
       </c>
     </row>
@@ -1994,179 +1768,6 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="31.83" customWidth="1" min="1" max="1"/>
-    <col width="63.66" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="B1" s="9" t="inlineStr">
-        <is>
-          <t>[DEF-034] Operar sobre la suscripción de otro usuario responde HTTP 500 en lugar de 404</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="75" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>Description / Overview</t>
-        </is>
-      </c>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>Cuando un usuario llama a pause_subscription, resume_subscription, cancel_subscription o update_subscription con el identificador de una suscripción de otro usuario, la API rechaza la operación (P0002 «Suscripción no encontrada») pero con HTTP 500 en lugar de 404.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>Reproduction Steps</t>
-        </is>
-      </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>1- Crear dos usuarios de prueba, A y B, con la configuración inicial salteada, y obtener el token de cada uno (PR-04).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>2- Con el token de B, crear una suscripción (POST /rest/v1/rpc/create_subscription) y guardar su id.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>3- Con el token de A, enviar POST /rest/v1/rpc/pause_subscription con body {"p_subscription_id":"&lt;id de B&gt;"}.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>4- Mirar el código HTTP y el cuerpo. Repetir con resume_subscription (sobre una pausada), cancel_subscription y update_subscription.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>Expected Behavior</t>
-        </is>
-      </c>
-      <c r="B10" s="11" t="inlineStr">
-        <is>
-          <t>Los casos esperan HTTP 404 con "code": "P0002" y "message": "Suscripción no encontrada".</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="60" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>Actual Behavior</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>HTTP 500 con {"code":"P0002","details":null,"hint":null,"message":"Suscripción no encontrada"}. El código y el mensaje coinciden; cambia el HTTP. La suscripción de B no se modifica.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>Incidence / Severity / Probability of reproduction</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>Severidad Baja - la operación se rechaza bien y no se filtra ningún dato, pero un «no encontrado» se informa como error del servidor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="15" customHeight="1">
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>100 % (4 de 4 ejecuciones).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="45" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>Story and Acceptance Criteria affected</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>US-56 · CA-9, US-57 · CA-7, US-58 · CA-9: «otro usuario recibe P0002 "Suscripción no encontrada"»; los casos agregan el HTTP 404.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t>Browsers tested</t>
-        </is>
-      </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>No aplica: llamada directa a la API.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="45" customHeight="1">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>Environment</t>
-        </is>
-      </c>
-      <c r="B21" s="11" t="inlineStr">
-        <is>
-          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63) · Edge Functions locales levantadas</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="225" customHeight="1">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="B23" s="11" t="inlineStr">
-        <is>
-          <t>- Defect ID: DEF-034
-- Estado: Abierto · se reproduce el 2026-10-27
-- Issue de GitHub: sin issue
-- Caso de prueba: CP-SUS-094, CP-SUS-100, CP-SUS-107 y CP-SUS-129
-- Encontrado en: ejecución de CP-SUS-094, 100, 107 y 129 (Entrega 2).
-- Reportó: Claude Code (IA), supervisado por Santiago
-- Evidencia: Respuesta de la API en las corridas de CP-SUS-094, 100, 107 y 129
-- Causa probable: PostgREST solo traduce a 4xx algunos códigos de error y P0002 no está entre ellos; hace falta un código propio (por ejemplo PT404) en la función. No se investigó a fondo ni se corrigió nada. Decisión pendiente: cambiar la función o el resultado esperado de los casos.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2312,11 +1913,11 @@
           <t>- Defect ID: DEF-035
 - Estado: Abierto · se reproduce el 2026-10-27
 - Issue de GitHub: sin issue
-- Caso de prueba: CP-SUS-065, CP-SUS-066, CP-SUS-095, CP-SUS-101, CP-SUS-108 y CP-SUS-130
-- Encontrado en: ejecución de CP-SUS-065, 066, 095, 101, 108 y 130 (Entrega 2).
+- Caso de prueba: CP-SUS-022 (otros cinco casos con el mismo defecto se recortaron del catálogo el 2026-10-27)
+- Encontrado en: ejecución de CP-SUS-022 y de otros cinco casos equivalentes (Entrega 2).
 - Reportó: Claude Code (IA), supervisado por Santiago
 - Evidencia: Respuesta de la API en las corridas de los seis casos
-- Parece un error de los casos: PostgREST responde 401 al rol anónimo (el mismo comportamiento se vio en CP-DEU-029 y CP-DEU-108). No se corrigió nada. Decisión pendiente: corregir el HTTP esperado en los seis casos.</t>
+- Parece un error de los casos: PostgREST responde 401 al rol anónimo (el mismo comportamiento se vio en otros casos que se recortaron del catálogo el 2026-10-27). No se corrigió nada. Decisión pendiente: corregir el HTTP esperado en el caso.</t>
         </is>
       </c>
     </row>
@@ -2325,7 +1926,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2396,7 +1997,7 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>La fila del mes con tipo de cambio tiene data-blocked="false" y la del mes sin tipo de cambio data-blocked="true" (CP-SUS-157, paso 11).</t>
+          <t>La fila del mes con tipo de cambio tiene data-blocked="false" y la del mes sin tipo de cambio data-blocked="true" (CP-SUS-048, paso 11).</t>
         </is>
       </c>
     </row>
@@ -2478,11 +2079,191 @@
           <t>- Defect ID: DEF-036
 - Estado: Abierto · se reproduce el 2026-10-27
 - Issue de GitHub: sin issue
-- Caso de prueba: CP-SUS-157
-- Encontrado en: ejecución de CP-SUS-157 (Entrega 2).
+- Caso de prueba: CP-SUS-048
+- Encontrado en: ejecución de CP-SUS-048 (Entrega 2).
 - Reportó: Claude Code (IA), supervisado por Santiago
-- Evidencia: Observaciones de la corrida de CP-SUS-157
+- Evidencia: Observaciones de la corrida de CP-SUS-048
 - En src/components/subscriptions/SubscriptionPreview.tsx el atributo se escribe como data-blocked={row.blockedBy ? 'true' : undefined}. Parece un error del caso, o un atributo de automatización por completar. No se corrigió nada.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31.83" customWidth="1" min="1" max="1"/>
+    <col width="63.66" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="45" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>[DEF-037] El primer clic en «US$» de «Nueva deuda» se pierde: el error de «Persona» corre los botones y la moneda no se selecciona</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Description / Overview</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>En «Nueva deuda», si el primer clic sobre el formulario es en «US$», la moneda no se selecciona y no aparece el campo «Tipo de cambio (ARS por US$)». Hace falta un segundo clic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Reproduction Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>1- Abrir la app e iniciar sesión con un usuario de prueba (con la configuración inicial salteada).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>2- Abrir /debts/new (Deudas → «Nueva deuda»): el foco queda en «Persona».</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>3- Sin escribir nada, hacer clic en «US$».</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>4- Mirar el formulario: la moneda sigue sin cambiar, no aparece el campo «Tipo de cambio (ARS por US$)» y debajo de «Persona» aparece «Ingresá el nombre de la persona».</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>5- Hacer clic otra vez en «US$»: ahora sí se selecciona y aparece el campo «Tipo de cambio».</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Expected Behavior</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>CP-DEU-024 (paso 6): al hacer clic en «US$» se selecciona la moneda y aparece el campo «Tipo de cambio (ARS por US$)».</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Actual Behavior</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>El primer clic en «US$» no hace nada visible. Al salir del foco de «Persona» aparece el error «Ingresá el nombre de la persona» y los botones bajan unos 26 px (la caja de «US$» pasa de y = 343,8 a y = 370,0 entre apretar y soltar el botón del mouse), así que el clic cae en otro elemento. El segundo clic funciona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Incidence / Severity / Probability of reproduction</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Severidad Media - no se pierden datos y con un segundo clic se puede seguir, pero quien carga una deuda en dólares piensa que la moneda no funciona o que falta el campo del tipo de cambio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>100 % (3 de 3 ejecuciones).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Story and Acceptance Criteria affected</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>US-36 · CA-6: cargar una deuda suelta en US$ con tipo de cambio (CP-DEU-024, paso 6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Browsers tested</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Chromium (Playwright 1.63), ventana de 420 × 900. No se probó en otros navegadores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="225" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>- Defect ID: DEF-037
+- Estado: Abierto · se reproduce el 2026-10-27
+- Issue de GitHub: sin issue
+- Caso de prueba: CP-DEU-024
+- Encontrado en: ejecución de CP-DEU-024 (Entrega 2).
+- Reportó: Claude Code (IA), supervisado por Santiago
+- Evidencia: Medidas de la corrida de CP-DEU-024 (posición de «US$» antes y después de apretar el mouse)
+- Causa probable: la validación al perder el foco muestra el mensaje de error entre el mousedown y el mouseup y desplaza los botones, de modo que el clic no llega al botón. No se corrigió nada. Con un segundo clic el resto del caso se cumple (≈ $0,01 y se guarda amount 0.01, fx_rate 0.5000 y amount_ars 0.01). Puede explicar parte de las dudas del equipo sobre los casos de tipo de cambio en US$ (dos casos recortados del catálogo).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(ejecucion): suma los 8 casos de Deudas que faltaban ejecutar (CP-DEU-001, 002, 003, 004, 011, 012, 013 y 025)
Se ejecutaron con Playwright contra Vite + Supabase local: 2 PASSED (004 y 012),
4 DUDA (001, 002, 003 y 011), 1 FAILED (025, DEF-037) y 1 BLOCKED (013, US-82).
Los DUDA salen de pasos que faltan o están mal ordenados en los casos (no piden
elegir cuenta, fijan el tipo de cambio antes de cambiar el mes) y de los
parámetros de una sola persona, porque la función de varias personas no existe.

Se actualizan 04, 05 (DEF-037 suma CP-DEU-025), 06, README y los tres Excel:
197 casos con resultado (180 PASSED, 9 FAILED, 4 DUDA, 4 BLOCKED).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega-2/05-reportes-de-defectos.xlsx
+++ b/entrega-2/05-reportes-de-defectos.xlsx
@@ -842,7 +842,7 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>CP-DEU-024</t>
+          <t>CP-DEU-024 y CP-DEU-025</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
@@ -906,6 +906,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -918,6 +919,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -958,6 +960,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -970,6 +973,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="60" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -982,6 +986,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
@@ -1001,6 +1006,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="60" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
@@ -1013,6 +1019,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -1025,6 +1032,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
@@ -1037,6 +1045,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="240" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
@@ -1086,6 +1095,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1098,6 +1108,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1138,6 +1149,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -1150,6 +1162,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -1162,6 +1175,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
@@ -1181,6 +1195,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
@@ -1193,6 +1208,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -1205,6 +1221,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
@@ -1217,6 +1234,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="240" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
@@ -1266,6 +1284,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1278,6 +1297,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1318,6 +1338,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -1330,6 +1351,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -1342,6 +1364,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
@@ -1361,6 +1384,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
@@ -1373,6 +1397,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -1385,6 +1410,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
@@ -1397,6 +1423,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="180" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
@@ -1446,6 +1473,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="75" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1458,6 +1486,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1491,6 +1520,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
@@ -1503,6 +1533,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -1515,6 +1546,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
@@ -1534,6 +1566,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
@@ -1546,6 +1579,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
@@ -1558,6 +1592,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
@@ -1570,6 +1605,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="165" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
@@ -1619,6 +1655,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="75" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1631,6 +1668,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1664,6 +1702,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
@@ -1676,6 +1715,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -1688,6 +1728,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
@@ -1707,6 +1748,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
@@ -1719,6 +1761,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
@@ -1731,6 +1774,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
@@ -1743,6 +1787,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="225" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
@@ -1792,6 +1837,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1804,6 +1850,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1823,6 +1870,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
@@ -1835,6 +1883,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
@@ -1847,6 +1896,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -1866,6 +1916,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
@@ -1878,6 +1929,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
@@ -1890,6 +1942,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" ht="45" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
@@ -1902,6 +1955,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="210" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
@@ -1951,6 +2005,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1963,6 +2018,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1989,6 +2045,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
@@ -2001,6 +2058,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -2013,6 +2071,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -2032,6 +2091,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
@@ -2044,6 +2104,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
@@ -2056,6 +2117,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="45" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -2068,6 +2130,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="165" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
@@ -2117,6 +2180,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -2129,6 +2193,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -2169,6 +2234,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -2181,6 +2247,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -2193,6 +2260,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="60" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
@@ -2212,6 +2280,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
@@ -2224,6 +2293,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -2236,6 +2306,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
@@ -2248,6 +2319,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="225" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
@@ -2259,11 +2331,11 @@
           <t>- Defect ID: DEF-037
 - Estado: Abierto · se reproduce el 2026-10-27
 - Issue de GitHub: sin issue
-- Caso de prueba: CP-DEU-024
-- Encontrado en: ejecución de CP-DEU-024 (Entrega 2).
+- Caso de prueba: CP-DEU-024 y CP-DEU-025
+- Encontrado en: ejecución de CP-DEU-024 y CP-DEU-025 (Entrega 2).
 - Reportó: Claude Code (IA), supervisado por Santiago
 - Evidencia: Medidas de la corrida de CP-DEU-024 (posición de «US$» antes y después de apretar el mouse)
-- Causa probable: la validación al perder el foco muestra el mensaje de error entre el mousedown y el mouseup y desplaza los botones, de modo que el clic no llega al botón. No se corrigió nada. Con un segundo clic el resto del caso se cumple (≈ $0,01 y se guarda amount 0.01, fx_rate 0.5000 y amount_ars 0.01). Puede explicar parte de las dudas del equipo sobre los casos de tipo de cambio en US$ (dos casos recortados del catálogo).</t>
+- Causa probable: la validación al perder el foco muestra el mensaje de error entre el mousedown y el mouseup y desplaza los botones, de modo que el clic no llega al botón. No se corrigió nada. Con un segundo clic el resto del caso se cumple (≈ $0,01 y se guarda amount 0.01, fx_rate 0.5000 y amount_ars 0.01). Puede explicar parte de las dudas del equipo sobre los casos de tipo de cambio en US$ (dos casos recortados del catálogo). Se reprodujo también en CP-DEU-025 (2026-10-27), con el mismo comportamiento al hacer clic en «US$» apenas se abre «Nueva deuda»; con un segundo clic el resto del caso se cumple.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(entrega-2): guía para la defensa, gráficos de resultados y DEF-036 en US-75
La consigna pide un gráfico con los porcentajes de PASSED, FAILED y BLOCKED, y el 06 lo
mencionaba pero la planilla no tenía ninguno: se suman dos gráficos SVG (por entrega y por
módulo de V2). La guía junta el mapa de la consigna, los casos que cambiaron de estado y qué
caso abrir para cada tema. DEF-036 apuntaba a US-61, pero la vista previa es US-75 · CA-6.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega-2/05-reportes-de-defectos.xlsx
+++ b/entrega-2/05-reportes-de-defectos.xlsx
@@ -810,7 +810,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>US-61 · Vista previa del calendario al dar de alta una suscripción</t>
+          <t>US-75 · Vista previa del calendario al dar de alta una suscripción</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -906,7 +906,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -919,7 +918,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -960,7 +958,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -973,7 +970,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="60" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -986,7 +982,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
@@ -1006,7 +1001,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="60" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
@@ -1019,7 +1013,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -1032,7 +1025,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
@@ -1045,7 +1037,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24" ht="240" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
@@ -1095,7 +1086,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1108,7 +1098,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1149,7 +1138,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -1162,7 +1150,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -1175,7 +1162,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
@@ -1195,7 +1181,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
@@ -1208,7 +1193,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -1221,7 +1205,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
@@ -1234,7 +1217,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24" ht="240" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
@@ -1284,7 +1266,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1297,7 +1278,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1338,7 +1318,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -1351,7 +1330,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -1364,7 +1342,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
@@ -1384,7 +1361,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
@@ -1397,7 +1373,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -1410,7 +1385,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
@@ -1423,7 +1397,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24" ht="180" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
@@ -1473,7 +1446,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="75" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1486,7 +1458,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1520,7 +1491,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
@@ -1533,7 +1503,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -1546,7 +1515,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
@@ -1566,7 +1534,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
@@ -1579,7 +1546,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
@@ -1592,7 +1558,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
@@ -1605,7 +1570,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="165" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
@@ -1655,7 +1619,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="75" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1668,7 +1631,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1702,7 +1664,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
@@ -1715,7 +1676,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -1728,7 +1688,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
@@ -1748,7 +1707,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
@@ -1761,7 +1719,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
@@ -1774,7 +1731,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
@@ -1787,7 +1743,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="225" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
@@ -1837,7 +1792,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1850,7 +1804,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1870,7 +1823,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
@@ -1883,7 +1835,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
@@ -1896,7 +1847,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -1916,7 +1866,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
@@ -1929,7 +1878,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
@@ -1942,7 +1890,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19" ht="45" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
@@ -1955,7 +1902,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21" ht="210" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
@@ -2005,7 +1951,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -2018,7 +1963,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -2045,7 +1989,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
@@ -2058,7 +2001,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -2071,7 +2013,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -2091,7 +2032,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
@@ -2100,11 +2040,10 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>US-61 · CA-5 (vista previa con meses bloqueados por falta de tipo de cambio).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
+          <t>US-75 · CA-6 (vista previa con meses bloqueados por falta de tipo de cambio).</t>
+        </is>
+      </c>
+    </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
@@ -2117,7 +2056,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="45" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -2130,7 +2068,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="165" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
@@ -2180,7 +2117,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -2193,7 +2129,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -2234,7 +2169,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -2247,7 +2181,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -2260,7 +2193,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="60" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
@@ -2280,7 +2212,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
@@ -2293,7 +2224,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -2306,7 +2236,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
@@ -2319,7 +2248,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24" ht="225" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(entrega-2): saca los nombres de responsables de los reportes de ejecución y de defectos
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega-2/05-reportes-de-defectos.xlsx
+++ b/entrega-2/05-reportes-de-defectos.xlsx
@@ -906,6 +906,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -918,6 +919,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -958,6 +960,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -970,6 +973,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="60" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -982,6 +986,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
@@ -1001,6 +1006,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="60" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
@@ -1013,6 +1019,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -1025,6 +1032,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
@@ -1037,6 +1045,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="240" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
@@ -1050,7 +1059,7 @@
 - Issue de GitHub: sin issue
 - Caso de prueba: CP-EXP-027
 - Encontrado en: ejecución de CP-EXP-027 (Entrega 2).
-- Reportó: Claude Code (IA), supervisado por Santiago
+- Reportó: Claude Code (IA)
 - Evidencia: Observado en la corrida de CP-EXP-027: la hoja sigue abierta tras el clic; document.elementFromPoint(5, 5) = DIV.fixed.inset-0.-z-10.bg-[rgba(43,30,25,0.32)], aria-hidden=true
 - Causa probable: en src/components/transactions/ExportTransactionsDialog.tsx el cierre por clic exige e.target === e.currentTarget, pero el div de fondo es hijo del contenedor y cubre toda la pantalla: recibe el clic y el destino nunca coincide. No se corrigió nada.</t>
         </is>
@@ -1086,6 +1095,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1098,6 +1108,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1138,6 +1149,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -1150,6 +1162,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -1162,6 +1175,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
@@ -1181,6 +1195,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
@@ -1193,6 +1208,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -1205,6 +1221,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
@@ -1217,6 +1234,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="240" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
@@ -1230,7 +1248,7 @@
 - Issue de GitHub: sin issue
 - Caso de prueba: CP-EXP-028 (el caso equivalente con «Adelante» se recortó del catálogo el 2026-10-27)
 - Encontrado en: ejecución de CP-EXP-028 y de su caso equivalente con «Adelante» (Entrega 2).
-- Reportó: Claude Code (IA), supervisado por Santiago
+- Reportó: Claude Code (IA)
 - Evidencia: Observado en las corridas de CP-EXP-028 (y su caso equivalente con «Adelante», recortado): URL cambiada con la hoja abierta; log de popstate: ['popstate@?period=2026-08']
 - Causa no determinada. En ExportTransactionsDialog.tsx hay un efecto que cierra la hoja cuando cambia location.key y un oyente de popstate; ninguno logra cerrarla. Hipótesis sin confirmar: el efecto que reinicia initialLocationKeyRef cuando cambia location.key corre antes del que compara la clave y la deja siempre igual. No se corrigió nada.</t>
         </is>
@@ -1266,6 +1284,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1278,6 +1297,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1318,6 +1338,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -1330,6 +1351,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -1342,6 +1364,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
@@ -1361,6 +1384,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
@@ -1373,6 +1397,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -1385,6 +1410,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
@@ -1397,6 +1423,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="180" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
@@ -1410,7 +1437,7 @@
 - Issue de GitHub: sin issue
 - Caso de prueba: CP-EXP-029
 - Encontrado en: ejecución de CP-EXP-029 (Entrega 2).
-- Reportó: Claude Code (IA), supervisado por Santiago
+- Reportó: Claude Code (IA)
 - Evidencia: Observado en la corrida de CP-EXP-029: aviso de éxito en el período anterior; descargas registradas por el navegador = 1
 - Relacionado con DEF-031: el cierre por «Atrás» no llega a abortar la exportación en curso (AbortController). No se investigó a fondo. No se corrigió nada.</t>
         </is>
@@ -1446,6 +1473,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="75" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1458,6 +1486,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1491,6 +1520,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
@@ -1503,6 +1533,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -1515,6 +1546,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
@@ -1534,6 +1566,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
@@ -1546,6 +1579,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
@@ -1558,6 +1592,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
@@ -1570,6 +1605,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="165" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
@@ -1583,7 +1619,7 @@
 - Issue de GitHub: sin issue
 - Caso de prueba: CP-IMP-024
 - Encontrado en: ejecución de CP-IMP-024 (Entrega 2).
-- Reportó: Claude Code (IA), supervisado por Santiago
+- Reportó: Claude Code (IA)
 - Evidencia: Texto de la tarjeta import-row-2 en la corrida de CP-IMP-024
 - Causa probable: la tarjeta arma el detalle con el texto leído del archivo y no con el nombre del catálogo que resolvió la fila. No se investigó a fondo ni se corrigió nada.</t>
         </is>
@@ -1619,6 +1655,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="75" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1631,6 +1668,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1664,6 +1702,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
@@ -1676,6 +1715,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -1688,6 +1728,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
@@ -1707,6 +1748,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
@@ -1719,6 +1761,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
@@ -1731,6 +1774,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
@@ -1743,6 +1787,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="225" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
@@ -1756,7 +1801,7 @@
 - Issue de GitHub: sin issue
 - Caso de prueba: CP-SUS-032 (otros tres casos con el mismo defecto se recortaron del catálogo el 2026-10-27)
 - Encontrado en: ejecución de CP-SUS-032 y de otros tres casos equivalentes (Entrega 2).
-- Reportó: Claude Code (IA), supervisado por Santiago
+- Reportó: Claude Code (IA)
 - Evidencia: Respuesta de la API en las corridas de CP-SUS-032 y de otros tres casos equivalentes
 - Causa probable: PostgREST solo traduce a 4xx algunos códigos de error y P0002 no está entre ellos; hace falta un código propio (por ejemplo PT404) en la función. No se investigó a fondo ni se corrigió nada. Decisión pendiente: cambiar la función o el resultado esperado de los casos.</t>
         </is>
@@ -1792,6 +1837,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1804,6 +1850,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1823,6 +1870,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
@@ -1835,6 +1883,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
@@ -1847,6 +1896,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -1866,6 +1916,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
@@ -1878,6 +1929,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
@@ -1890,6 +1942,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" ht="45" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
@@ -1902,6 +1955,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="210" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
@@ -1915,7 +1969,7 @@
 - Issue de GitHub: sin issue
 - Caso de prueba: CP-SUS-022 (otros cinco casos con el mismo defecto se recortaron del catálogo el 2026-10-27)
 - Encontrado en: ejecución de CP-SUS-022 y de otros cinco casos equivalentes (Entrega 2).
-- Reportó: Claude Code (IA), supervisado por Santiago
+- Reportó: Claude Code (IA)
 - Evidencia: Respuesta de la API en las corridas de los seis casos
 - Parece un error de los casos: PostgREST responde 401 al rol anónimo (el mismo comportamiento se vio en otros casos que se recortaron del catálogo el 2026-10-27). No se corrigió nada. Decisión pendiente: corregir el HTTP esperado en el caso.</t>
         </is>
@@ -1951,6 +2005,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1963,6 +2018,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -1989,6 +2045,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
@@ -2001,6 +2058,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -2013,6 +2071,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -2032,6 +2091,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
@@ -2044,6 +2104,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
@@ -2056,6 +2117,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="45" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -2068,6 +2130,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="165" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
@@ -2081,7 +2144,7 @@
 - Issue de GitHub: sin issue
 - Caso de prueba: CP-SUS-048
 - Encontrado en: ejecución de CP-SUS-048 (Entrega 2).
-- Reportó: Claude Code (IA), supervisado por Santiago
+- Reportó: Claude Code (IA)
 - Evidencia: Observaciones de la corrida de CP-SUS-048
 - En src/components/subscriptions/SubscriptionPreview.tsx el atributo se escribe como data-blocked={row.blockedBy ? 'true' : undefined}. Parece un error del caso, o un atributo de automatización por completar. No se corrigió nada.</t>
         </is>
@@ -2117,6 +2180,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -2129,6 +2193,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -2169,6 +2234,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -2181,6 +2247,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -2193,6 +2260,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="60" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
@@ -2212,6 +2280,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
@@ -2224,6 +2293,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -2236,6 +2306,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
@@ -2248,6 +2319,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="225" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
@@ -2261,7 +2333,7 @@
 - Issue de GitHub: sin issue
 - Caso de prueba: CP-DEU-024 y CP-DEU-025
 - Encontrado en: ejecución de CP-DEU-024 y CP-DEU-025 (Entrega 2).
-- Reportó: Claude Code (IA), supervisado por Santiago
+- Reportó: Claude Code (IA)
 - Evidencia: Medidas de la corrida de CP-DEU-024 (posición de «US$» antes y después de apretar el mouse)
 - Causa probable: la validación al perder el foco muestra el mensaje de error entre el mousedown y el mouseup y desplaza los botones, de modo que el clic no llega al botón. No se corrigió nada. Con un segundo clic el resto del caso se cumple (≈ $0,01 y se guarda amount 0.01, fx_rate 0.5000 y amount_ars 0.01). Puede explicar parte de las dudas del equipo sobre los casos de tipo de cambio en US$ (dos casos recortados del catálogo). Se reprodujo también en CP-DEU-025 (2026-10-27), con el mismo comportamiento al hacer clic en «US$» apenas se abre «Nueva deuda»; con un segundo clic el resto del caso se cumple.</t>
         </is>

</xml_diff>

<commit_message>
docs(entrega-2): funde el reporte de ejecución (06) en la ejecución (04)
El 06 solo agregaba resumen, cobertura, defectos abiertos, criterios de salida y
desvíos sobre el registro por caso del 04, y obligaba a mantener el mismo registro
en dos lugares. Pasa a ser la sección «Reporte de ejecución» de 04-ejecucion.md y
el pie de la hoja «Índice» de 04-ejecucion.xlsx. Se borran 06-reporte-de-ejecucion.md
y .xlsx y se actualizan el README, la guía de la defensa, el ADR-027 y las demás
referencias.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega-2/05-reportes-de-defectos.xlsx
+++ b/entrega-2/05-reportes-de-defectos.xlsx
@@ -1028,7 +1028,7 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Chromium (Playwright 1.63), ventana de 420 × 900. No se probó en otros navegadores.</t>
+          <t>Chromium, ventana de 420 × 900. No se probó en otros navegadores.</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63), reloj fijado en 09/10/2026</t>
+          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium, reloj fijado en 09/10/2026</t>
         </is>
       </c>
     </row>
@@ -1059,7 +1059,6 @@
 - Issue de GitHub: sin issue
 - Caso de prueba: CP-EXP-027
 - Encontrado en: ejecución de CP-EXP-027 (Entrega 2).
-- Reportó: Claude Code (IA)
 - Evidencia: Observado en la corrida de CP-EXP-027: la hoja sigue abierta tras el clic; document.elementFromPoint(5, 5) = DIV.fixed.inset-0.-z-10.bg-[rgba(43,30,25,0.32)], aria-hidden=true
 - Causa probable: en src/components/transactions/ExportTransactionsDialog.tsx el cierre por clic exige e.target === e.currentTarget, pero el div de fondo es hijo del contenedor y cubre toda la pantalla: recibe el clic y el destino nunca coincide. No se corrigió nada.</t>
         </is>
@@ -1217,7 +1216,7 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Chromium (Playwright 1.63). No se probó en otros navegadores.</t>
+          <t>Chromium. No se probó en otros navegadores.</t>
         </is>
       </c>
     </row>
@@ -1230,7 +1229,7 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63), reloj fijado en 09/10/2026</t>
+          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium, reloj fijado en 09/10/2026</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1247,6 @@
 - Issue de GitHub: sin issue
 - Caso de prueba: CP-EXP-028 (el caso equivalente con «Adelante» se recortó del catálogo el 2026-10-27)
 - Encontrado en: ejecución de CP-EXP-028 y de su caso equivalente con «Adelante» (Entrega 2).
-- Reportó: Claude Code (IA)
 - Evidencia: Observado en las corridas de CP-EXP-028 (y su caso equivalente con «Adelante», recortado): URL cambiada con la hoja abierta; log de popstate: ['popstate@?period=2026-08']
 - Causa no determinada. En ExportTransactionsDialog.tsx hay un efecto que cierra la hoja cuando cambia location.key y un oyente de popstate; ninguno logra cerrarla. Hipótesis sin confirmar: el efecto que reinicia initialLocationKeyRef cuando cambia location.key corre antes del que compara la clave y la deja siempre igual. No se corrigió nada.</t>
         </is>
@@ -1320,7 +1318,7 @@
     <row r="7" ht="45" customHeight="1">
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>3- Demorar unos segundos las respuestas de /rest/v1/transactions (en las pruebas, 3 s con Playwright; en DevTools, «1 kbit/s» y latencia 2000 ms).</t>
+          <t>3- Demorar unos segundos las respuestas de /rest/v1/transactions (en las pruebas, 3 s; en DevTools, «1 kbit/s» y latencia 2000 ms).</t>
         </is>
       </c>
     </row>
@@ -1406,7 +1404,7 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Chromium (Playwright 1.63). No se probó en otros navegadores.</t>
+          <t>Chromium. No se probó en otros navegadores.</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1417,7 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63), reloj fijado en 09/10/2026</t>
+          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium, reloj fijado en 09/10/2026</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1435,6 @@
 - Issue de GitHub: sin issue
 - Caso de prueba: CP-EXP-029
 - Encontrado en: ejecución de CP-EXP-029 (Entrega 2).
-- Reportó: Claude Code (IA)
 - Evidencia: Observado en la corrida de CP-EXP-029: aviso de éxito en el período anterior; descargas registradas por el navegador = 1
 - Relacionado con DEF-031: el cierre por «Atrás» no llega a abortar la exportación en curso (AbortController). No se investigó a fondo. No se corrigió nada.</t>
         </is>
@@ -1588,7 +1585,7 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Chromium (Playwright 1.63). No se probó en otros navegadores.</t>
+          <t>Chromium. No se probó en otros navegadores.</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1598,7 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63)</t>
+          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium</t>
         </is>
       </c>
     </row>
@@ -1619,7 +1616,6 @@
 - Issue de GitHub: sin issue
 - Caso de prueba: CP-IMP-024
 - Encontrado en: ejecución de CP-IMP-024 (Entrega 2).
-- Reportó: Claude Code (IA)
 - Evidencia: Texto de la tarjeta import-row-2 en la corrida de CP-IMP-024
 - Causa probable: la tarjeta arma el detalle con el texto leído del archivo y no con el nombre del catálogo que resolvió la fila. No se investigó a fondo ni se corrigió nada.</t>
         </is>
@@ -1783,7 +1779,7 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63) · Edge Functions locales levantadas</t>
+          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium · Edge Functions locales levantadas</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1797,6 @@
 - Issue de GitHub: sin issue
 - Caso de prueba: CP-SUS-032 (otros tres casos con el mismo defecto se recortaron del catálogo el 2026-10-27)
 - Encontrado en: ejecución de CP-SUS-032 y de otros tres casos equivalentes (Entrega 2).
-- Reportó: Claude Code (IA)
 - Evidencia: Respuesta de la API en las corridas de CP-SUS-032 y de otros tres casos equivalentes
 - Causa probable: PostgREST solo traduce a 4xx algunos códigos de error y P0002 no está entre ellos; hace falta un código propio (por ejemplo PT404) en la función. No se investigó a fondo ni se corrigió nada. Decisión pendiente: cambiar la función o el resultado esperado de los casos.</t>
         </is>
@@ -1951,7 +1946,7 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63) · Edge Functions locales levantadas</t>
+          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium · Edge Functions locales levantadas</t>
         </is>
       </c>
     </row>
@@ -1969,7 +1964,6 @@
 - Issue de GitHub: sin issue
 - Caso de prueba: CP-SUS-022 (otros cinco casos con el mismo defecto se recortaron del catálogo el 2026-10-27)
 - Encontrado en: ejecución de CP-SUS-022 y de otros cinco casos equivalentes (Entrega 2).
-- Reportó: Claude Code (IA)
 - Evidencia: Respuesta de la API en las corridas de los seis casos
 - Parece un error de los casos: PostgREST responde 401 al rol anónimo (el mismo comportamiento se vio en otros casos que se recortaron del catálogo el 2026-10-27). No se corrigió nada. Decisión pendiente: corregir el HTTP esperado en el caso.</t>
         </is>
@@ -2113,7 +2107,7 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Chromium (Playwright 1.63). No se probó en otros navegadores.</t>
+          <t>Chromium. No se probó en otros navegadores.</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2120,7 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63) · Edge Functions locales levantadas</t>
+          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium · Edge Functions locales levantadas</t>
         </is>
       </c>
     </row>
@@ -2144,7 +2138,6 @@
 - Issue de GitHub: sin issue
 - Caso de prueba: CP-SUS-048
 - Encontrado en: ejecución de CP-SUS-048 (Entrega 2).
-- Reportó: Claude Code (IA)
 - Evidencia: Observaciones de la corrida de CP-SUS-048
 - En src/components/subscriptions/SubscriptionPreview.tsx el atributo se escribe como data-blocked={row.blockedBy ? 'true' : undefined}. Parece un error del caso, o un atributo de automatización por completar. No se corrigió nada.</t>
         </is>
@@ -2302,7 +2295,7 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Chromium (Playwright 1.63), ventana de 420 × 900. No se probó en otros navegadores.</t>
+          <t>Chromium, ventana de 420 × 900. No se probó en otros navegadores.</t>
         </is>
       </c>
     </row>
@@ -2315,7 +2308,7 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium (Playwright 1.63)</t>
+          <t>Local, 2026-10-27 · Vite (http://127.0.0.1:5173) + Supabase local · main 1c72d0f · Chromium</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2326,6 @@
 - Issue de GitHub: sin issue
 - Caso de prueba: CP-DEU-024 y CP-DEU-025
 - Encontrado en: ejecución de CP-DEU-024 y CP-DEU-025 (Entrega 2).
-- Reportó: Claude Code (IA)
 - Evidencia: Medidas de la corrida de CP-DEU-024 (posición de «US$» antes y después de apretar el mouse)
 - Causa probable: la validación al perder el foco muestra el mensaje de error entre el mousedown y el mouseup y desplaza los botones, de modo que el clic no llega al botón. No se corrigió nada. Con un segundo clic el resto del caso se cumple (≈ $0,01 y se guarda amount 0.01, fx_rate 0.5000 y amount_ars 0.01). Puede explicar parte de las dudas del equipo sobre los casos de tipo de cambio en US$ (dos casos recortados del catálogo). Se reprodujo también en CP-DEU-025 (2026-10-27), con el mismo comportamiento al hacer clic en «US$» apenas se abre «Nueva deuda»; con un segundo clic el resto del caso se cumple.</t>
         </is>

</xml_diff>